<commit_message>
added expanse mnemonic logic but will be updated again
</commit_message>
<xml_diff>
--- a/Filtered_V3.0/COCAT_HCAFloridaAventura.xlsx
+++ b/Filtered_V3.0/COCAT_HCAFloridaAventura.xlsx
@@ -618,7 +618,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3M (360 Encompass)-Abstracting </t>
+          <t>3M (360 Encompass)-ABSDPI</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -700,7 +700,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve">3M (360 Encompass)-Admissions </t>
+          <t>3M (360 Encompass)-ADMO</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -782,7 +782,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t xml:space="preserve">3M (360 Encompass)-Charges </t>
+          <t>3M (360 Encompass)-ITSDIRO</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -827,22 +827,22 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Inbound</t>
+          <t>Outbound</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Patient Accounting</t>
+          <t>ITSDIRO</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>DFT</t>
+          <t>ORU</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Charges </t>
+          <t xml:space="preserve">ITS DI Results </t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve">3M (360 Encompass)-ITS DI Results </t>
+          <t>3M (360 Encompass)-ITSHMRO</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -914,7 +914,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>ITSDIRO</t>
+          <t>ITSHMRO</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -924,7 +924,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t xml:space="preserve">ITS DI Results </t>
+          <t xml:space="preserve">ITS HM Results </t>
         </is>
       </c>
     </row>
@@ -946,7 +946,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t xml:space="preserve">3M (360 Encompass)-ITS HM Results </t>
+          <t>3M (360 Encompass)-ITSHMRO</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Outbound</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3M (360 Encompass)-ITS HM Results </t>
+          <t>3M (360 Encompass)-LABRES</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1073,12 +1073,12 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Inbound</t>
+          <t>Outbound</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>ITSHMRO</t>
+          <t>LABRES</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1088,7 +1088,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ITS HM Results </t>
+          <t xml:space="preserve">Lab Results (Discrete) </t>
         </is>
       </c>
     </row>
@@ -1110,7 +1110,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t xml:space="preserve">3M (360 Encompass)-Lab Results (Discrete) </t>
+          <t>3M (360 Encompass)-OMORDO</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1160,17 +1160,17 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>LABRES</t>
+          <t>OMORDO</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>ORU</t>
+          <t>iPeople OM Orders</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lab Results (Discrete) </t>
+          <t>ORM - iPeople</t>
         </is>
       </c>
     </row>
@@ -1192,7 +1192,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t xml:space="preserve">3M (360 Encompass)-OM Orders </t>
+          <t>3M (360 Encompass)-Patient Accounting</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1237,22 +1237,22 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Outbound</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>OMORDO</t>
+          <t>Patient Accounting</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>iPeople OM Orders</t>
+          <t>DFT</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>ORM - iPeople</t>
+          <t xml:space="preserve">Charges </t>
         </is>
       </c>
     </row>
@@ -1274,7 +1274,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>3M (360 Encompass)-iPeople ED Patient Visit Data</t>
+          <t>3M (360 Encompass)-iPeople EDM</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1356,7 +1356,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>3M (360 Encompass)-iPeople Medication Administration</t>
+          <t>3M (360 Encompass)-iPeople Meds</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1438,7 +1438,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>3M (360 Encompass)-iPeople Nursing Assessment Forms</t>
+          <t>3M (360 Encompass)-iPeople PCS</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t xml:space="preserve">AQuity Solutions (DocEP)-Admissions </t>
+          <t>AQuity Solutions (DocEP)-ADMO</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t xml:space="preserve">AQuity Solutions (DocEP)-ITS HM Results </t>
+          <t>AQuity Solutions (DocEP)-ITSHMRO</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Airstrip Technologies (ONE)-Admissions </t>
+          <t>Airstrip Technologies (ONE)-ADMO</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1952,7 +1952,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Alere (MAS RALS-Plus)-</t>
+          <t>Alere (MAS RALS-Plus)-ADMO</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1997,7 +1997,22 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>Inbound</t>
+          <t>Outbound</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>ADMO</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>ADT</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admissions </t>
         </is>
       </c>
     </row>
@@ -2019,7 +2034,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alere (MAS RALS-Plus)-Admissions </t>
+          <t>Alere (MAS RALS-Plus)-labpoc</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2064,22 +2079,7 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>Outbound</t>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>ADMO</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>ADT</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Admissions </t>
+          <t>Inbound</t>
         </is>
       </c>
     </row>
@@ -2163,7 +2163,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t xml:space="preserve">BD (Pyxis Medstation ES)-Admissions </t>
+          <t>BD (Pyxis Medstation ES)-ADMO</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2245,7 +2245,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t xml:space="preserve">BD (Pyxis Medstation ES)-Pharmacy Inventory </t>
+          <t>BD (Pyxis Medstation ES)-PHAINV</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2327,7 +2327,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t xml:space="preserve">BD (Pyxis Medstation ES)-Pharmacy Orders </t>
+          <t>BD (Pyxis Medstation ES)-PHAORD</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2471,7 +2471,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Computrition (Computrition)-Admissions </t>
+          <t>Computrition (Computrition)-ADMO</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2553,7 +2553,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Computrition (Computrition)-OM Orders </t>
+          <t>Computrition (Computrition)-OMORDO</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2697,7 +2697,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Datavant/CIOX (HealthSource to MPF-Patient Folder/HPF Facility)-</t>
+          <t>Datavant/CIOX (HealthSource to MPF-Patient Folder/HPF Facility)-imgurl</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2826,7 +2826,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dolbey (Fusion Voice)-Admissions </t>
+          <t>Dolbey (Fusion Voice)-ADMO</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2970,7 +2970,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Dolbey (Fusion)-</t>
+          <t>Dolbey (Fusion)-ITSDIRO</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -3015,7 +3015,22 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>Outbound</t>
+          <t>Inbound</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>ITSDIRO</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>ORU</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ITS DI Results </t>
         </is>
       </c>
     </row>
@@ -3037,7 +3052,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dolbey (Fusion)-ITS DI Results </t>
+          <t>Dolbey (Fusion)-radord</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -3082,22 +3097,7 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>Inbound</t>
-        </is>
-      </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>ITSDIRO</t>
-        </is>
-      </c>
-      <c r="R35" t="inlineStr">
-        <is>
-          <t>ORU</t>
-        </is>
-      </c>
-      <c r="S35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ITS DI Results </t>
+          <t>Outbound</t>
         </is>
       </c>
     </row>
@@ -3181,7 +3181,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Envision Healthcare (Envision Healthcare)-Admissions </t>
+          <t>Envision Healthcare (Envision Healthcare)-ADMO</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Envision Healthcare (Envision Healthcare)-ITS HM Results </t>
+          <t>Envision Healthcare (Envision Healthcare)-CWSO</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -3313,17 +3313,17 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>ITSHMRO</t>
+          <t>CWSO</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>ORU</t>
+          <t>SIU</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t xml:space="preserve">ITS HM Results </t>
+          <t xml:space="preserve">Scheduling </t>
         </is>
       </c>
     </row>
@@ -3345,7 +3345,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Envision Healthcare (Envision Healthcare)-ITS HM Results </t>
+          <t>Envision Healthcare (Envision Healthcare)-ITSHMRO</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -3390,7 +3390,7 @@
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>Inbound</t>
+          <t>Outbound</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Envision Healthcare (Envision Healthcare)-Scheduling </t>
+          <t>Envision Healthcare (Envision Healthcare)-ITSHMRO</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -3472,22 +3472,22 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>Outbound</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>CWSO</t>
+          <t>ITSHMRO</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>SIU</t>
+          <t>ORU</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scheduling </t>
+          <t xml:space="preserve">ITS HM Results </t>
         </is>
       </c>
     </row>
@@ -3509,7 +3509,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Envision Healthcare (Envision Healthcare)-iPeople ED Patient Visit Data</t>
+          <t>Envision Healthcare (Envision Healthcare)-iPeople EDM</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -3653,7 +3653,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Florida HIE (Event Notification Service)-Admissions </t>
+          <t>Florida HIE (Event Notification Service)-ADMO</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -3797,7 +3797,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t xml:space="preserve">GE (CMI - Carescape Gateway)-Admissions </t>
+          <t>GE (CMI - Carescape Gateway)-ADMO</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -3879,7 +3879,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t xml:space="preserve">GE (CMI - Carescape Gateway)-Scheduling </t>
+          <t>GE (CMI - Carescape Gateway)-CWSO</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -4023,7 +4023,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>GE (Centricity - CCG PACS)-</t>
+          <t>GE (Centricity - CCG PACS)-ADMO</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -4069,6 +4069,21 @@
       <c r="P48" t="inlineStr">
         <is>
           <t>Outbound</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>ADMO</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>ADT</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admissions </t>
         </is>
       </c>
     </row>
@@ -4090,7 +4105,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t xml:space="preserve">GE (Centricity - CCG PACS)-Admissions </t>
+          <t>GE (Centricity - CCG PACS)-ITSDIRO</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -4140,17 +4155,17 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>ADMO</t>
+          <t>ITSDIRO</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>ADT</t>
+          <t>ORU</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Admissions </t>
+          <t xml:space="preserve">ITS DI Results </t>
         </is>
       </c>
     </row>
@@ -4172,7 +4187,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t xml:space="preserve">GE (Centricity - CCG PACS)-ITS DI Results </t>
+          <t>GE (Centricity - CCG PACS)-ITSDIUI</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -4217,22 +4232,22 @@
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>Outbound</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>ITSDIRO</t>
+          <t>ITSDIUI</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>ORU</t>
+          <t>ORM</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t xml:space="preserve">ITS DI Results </t>
+          <t xml:space="preserve">Radiology Image Status </t>
         </is>
       </c>
     </row>
@@ -4254,7 +4269,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t xml:space="preserve">GE (Centricity - CCG PACS)-Radiology Image Status </t>
+          <t>GE (Centricity - CCG PACS)-ITSDIUI</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -4336,7 +4351,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t xml:space="preserve">GE (Centricity - CCG PACS)-Radiology Image Status </t>
+          <t>GE (Centricity - CCG PACS)-radord</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -4381,22 +4396,7 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>Inbound</t>
-        </is>
-      </c>
-      <c r="Q52" t="inlineStr">
-        <is>
-          <t>ITSDIUI</t>
-        </is>
-      </c>
-      <c r="R52" t="inlineStr">
-        <is>
-          <t>ORM</t>
-        </is>
-      </c>
-      <c r="S52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Radiology Image Status </t>
+          <t>Outbound</t>
         </is>
       </c>
     </row>
@@ -4480,7 +4480,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t xml:space="preserve">GE (Centricity Cardio Workflow-CCW to Centricity Cardio Workflow-CCW)-ITS HM Results </t>
+          <t>GE (Centricity Cardio Workflow-CCW to Centricity Cardio Workflow-CCW)-ITSHMRO</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>GE (Centricity Cardio Workflow-CCW to MPF-Patient Folder/HPF Facility)-</t>
+          <t>GE (Centricity Cardio Workflow-CCW to MPF-Patient Folder/HPF Facility)-imgurl</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -4753,7 +4753,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t xml:space="preserve">GE (Centricity Cardio Workflow-CCW)-Admissions </t>
+          <t>GE (Centricity Cardio Workflow-CCW)-ADMO</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -4835,7 +4835,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t xml:space="preserve">GE (Centricity Cardio Workflow-CCW)-Charges </t>
+          <t>GE (Centricity Cardio Workflow-CCW)-ITSHMRO</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -4885,17 +4885,17 @@
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>Patient Accounting</t>
+          <t>ITSHMRO</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>DFT</t>
+          <t>ORU</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Charges </t>
+          <t xml:space="preserve">ITS HM Results </t>
         </is>
       </c>
     </row>
@@ -4917,7 +4917,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t xml:space="preserve">GE (Centricity Cardio Workflow-CCW)-ITS HM Results </t>
+          <t>GE (Centricity Cardio Workflow-CCW)-OMORDO</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -4962,22 +4962,22 @@
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>Inbound</t>
+          <t>Outbound</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>ITSHMRO</t>
+          <t>OMORDO</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>ORU</t>
+          <t>ORM</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
         <is>
-          <t xml:space="preserve">ITS HM Results </t>
+          <t xml:space="preserve">OM Orders </t>
         </is>
       </c>
     </row>
@@ -4999,7 +4999,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t xml:space="preserve">GE (Centricity Cardio Workflow-CCW)-OM Orders </t>
+          <t>GE (Centricity Cardio Workflow-CCW)-Patient Accounting</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -5044,22 +5044,22 @@
       </c>
       <c r="P61" t="inlineStr">
         <is>
-          <t>Outbound</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>OMORDO</t>
+          <t>Patient Accounting</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>ORM</t>
+          <t>DFT</t>
         </is>
       </c>
       <c r="S61" t="inlineStr">
         <is>
-          <t xml:space="preserve">OM Orders </t>
+          <t xml:space="preserve">Charges </t>
         </is>
       </c>
     </row>
@@ -5143,7 +5143,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t xml:space="preserve">GE (Centricity MUSE to MPF-Patient Folder/HPF Facility)-ITS HM Results </t>
+          <t>GE (Centricity MUSE to MPF-Patient Folder/HPF Facility)-ITSHMRO</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -5287,7 +5287,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t xml:space="preserve">GE (Centricity MUSE)-Admissions </t>
+          <t>GE (Centricity MUSE)-ADMO</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -5369,7 +5369,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t xml:space="preserve">GE (Centricity MUSE)-Charges </t>
+          <t>GE (Centricity MUSE)-ITSHMRO</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -5419,17 +5419,17 @@
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>Patient Accounting</t>
+          <t>ITSHMRO</t>
         </is>
       </c>
       <c r="R66" t="inlineStr">
         <is>
-          <t>DFT</t>
+          <t>ORU</t>
         </is>
       </c>
       <c r="S66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Charges </t>
+          <t xml:space="preserve">ITS HM Results </t>
         </is>
       </c>
     </row>
@@ -5451,7 +5451,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t xml:space="preserve">GE (Centricity MUSE)-ITS HM Results </t>
+          <t>GE (Centricity MUSE)-OMORDO</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -5496,22 +5496,22 @@
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t>Inbound</t>
+          <t>Outbound</t>
         </is>
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>ITSHMRO</t>
+          <t>OMORDO</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
         <is>
-          <t>ORU</t>
+          <t>ORM</t>
         </is>
       </c>
       <c r="S67" t="inlineStr">
         <is>
-          <t xml:space="preserve">ITS HM Results </t>
+          <t xml:space="preserve">OM Orders </t>
         </is>
       </c>
     </row>
@@ -5533,7 +5533,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t xml:space="preserve">GE (Centricity MUSE)-OM Orders </t>
+          <t>GE (Centricity MUSE)-Patient Accounting</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -5578,22 +5578,22 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>Outbound</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>OMORDO</t>
+          <t>Patient Accounting</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>ORM</t>
+          <t>DFT</t>
         </is>
       </c>
       <c r="S68" t="inlineStr">
         <is>
-          <t xml:space="preserve">OM Orders </t>
+          <t xml:space="preserve">Charges </t>
         </is>
       </c>
     </row>
@@ -5677,7 +5677,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t xml:space="preserve">GE (Edison Datalogue to MPF-Patient Folder/HPF Facility)-ITS HM Results </t>
+          <t>GE (Edison Datalogue to MPF-Patient Folder/HPF Facility)-ITSHMRO</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -5821,7 +5821,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Google (Healthcare Data Engine - HDE)-</t>
+          <t>Google (Healthcare Data Engine - HDE)-ADMO</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -5867,6 +5867,21 @@
       <c r="P72" t="inlineStr">
         <is>
           <t>Outbound</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>ADMO</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>ADT</t>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admissions </t>
         </is>
       </c>
     </row>
@@ -5888,7 +5903,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t xml:space="preserve">Google (Healthcare Data Engine - HDE)-Admissions </t>
+          <t>Google (Healthcare Data Engine - HDE)-CWSO</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -5938,17 +5953,17 @@
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>ADMO</t>
+          <t>CWSO</t>
         </is>
       </c>
       <c r="R73" t="inlineStr">
         <is>
-          <t>ADT</t>
+          <t>iPeople Scheduling</t>
         </is>
       </c>
       <c r="S73" t="inlineStr">
         <is>
-          <t xml:space="preserve">Admissions </t>
+          <t>SIU</t>
         </is>
       </c>
     </row>
@@ -5970,7 +5985,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Google (Healthcare Data Engine - HDE)-ITS DI Results </t>
+          <t>Google (Healthcare Data Engine - HDE)-IMMUN</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -6020,17 +6035,17 @@
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>ITSDIRO</t>
+          <t>IMMUN</t>
         </is>
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>ORU</t>
+          <t>VXU</t>
         </is>
       </c>
       <c r="S74" t="inlineStr">
         <is>
-          <t xml:space="preserve">ITS DI Results </t>
+          <t>MU-Immunizations</t>
         </is>
       </c>
     </row>
@@ -6052,7 +6067,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Google (Healthcare Data Engine - HDE)-ITS HM Results </t>
+          <t>Google (Healthcare Data Engine - HDE)-ITSDIRO</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -6102,7 +6117,7 @@
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>ITSHMRO</t>
+          <t>ITSDIRO</t>
         </is>
       </c>
       <c r="R75" t="inlineStr">
@@ -6112,7 +6127,7 @@
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t xml:space="preserve">ITS HM Results </t>
+          <t xml:space="preserve">ITS DI Results </t>
         </is>
       </c>
     </row>
@@ -6134,7 +6149,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t xml:space="preserve">Google (Healthcare Data Engine - HDE)-Lab Results (Discrete) </t>
+          <t>Google (Healthcare Data Engine - HDE)-ITSHMRO</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -6184,7 +6199,7 @@
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>LABRES</t>
+          <t>ITSHMRO</t>
         </is>
       </c>
       <c r="R76" t="inlineStr">
@@ -6194,7 +6209,7 @@
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lab Results (Discrete) </t>
+          <t xml:space="preserve">ITS HM Results </t>
         </is>
       </c>
     </row>
@@ -6216,7 +6231,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Google (Healthcare Data Engine - HDE)-MU-Immunizations</t>
+          <t>Google (Healthcare Data Engine - HDE)-LABRES</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -6266,17 +6281,17 @@
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>IMMUN</t>
+          <t>LABRES</t>
         </is>
       </c>
       <c r="R77" t="inlineStr">
         <is>
-          <t>VXU</t>
+          <t>ORU</t>
         </is>
       </c>
       <c r="S77" t="inlineStr">
         <is>
-          <t>MU-Immunizations</t>
+          <t xml:space="preserve">Lab Results (Discrete) </t>
         </is>
       </c>
     </row>
@@ -6298,7 +6313,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Google (Healthcare Data Engine - HDE)-Pathology Results</t>
+          <t>Google (Healthcare Data Engine - HDE)-LABRES2</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -6380,7 +6395,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t xml:space="preserve">Google (Healthcare Data Engine - HDE)-Pharmacy Orders </t>
+          <t>Google (Healthcare Data Engine - HDE)-PHAORD</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -6462,7 +6477,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t xml:space="preserve">Google (Healthcare Data Engine - HDE)-Scheduling </t>
+          <t>Google (Healthcare Data Engine - HDE)-iPeople EDM</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -6512,17 +6527,17 @@
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>CWSO</t>
+          <t>iPeople EDM</t>
         </is>
       </c>
       <c r="R80" t="inlineStr">
         <is>
-          <t>iPeople Scheduling</t>
+          <t>EDM - iPeople</t>
         </is>
       </c>
       <c r="S80" t="inlineStr">
         <is>
-          <t>SIU</t>
+          <t>iPeople ED Patient Visit Data</t>
         </is>
       </c>
     </row>
@@ -6544,7 +6559,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Google (Healthcare Data Engine - HDE)-iPeople ED Patient Visit Data</t>
+          <t>Google (Healthcare Data Engine - HDE)-iPeople Meds</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -6594,17 +6609,17 @@
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>iPeople EDM</t>
+          <t>iPeople Meds</t>
         </is>
       </c>
       <c r="R81" t="inlineStr">
         <is>
-          <t>EDM - iPeople</t>
+          <t>RAS - iPeople</t>
         </is>
       </c>
       <c r="S81" t="inlineStr">
         <is>
-          <t>iPeople ED Patient Visit Data</t>
+          <t>iPeople Medication Administration</t>
         </is>
       </c>
     </row>
@@ -6626,7 +6641,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Google (Healthcare Data Engine - HDE)-iPeople Medication Administration</t>
+          <t>Google (Healthcare Data Engine - HDE)-iPeople PCS</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -6676,17 +6691,17 @@
       </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t>iPeople Meds</t>
+          <t>iPeople PCS</t>
         </is>
       </c>
       <c r="R82" t="inlineStr">
         <is>
-          <t>RAS - iPeople</t>
+          <t>PCS - iPeople</t>
         </is>
       </c>
       <c r="S82" t="inlineStr">
         <is>
-          <t>iPeople Medication Administration</t>
+          <t>iPeople Nursing Assessment Forms</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6723,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Google (Healthcare Data Engine - HDE)-iPeople Nursing Assessment Forms</t>
+          <t>Google (Healthcare Data Engine - HDE)-radord</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -6754,21 +6769,6 @@
       <c r="P83" t="inlineStr">
         <is>
           <t>Outbound</t>
-        </is>
-      </c>
-      <c r="Q83" t="inlineStr">
-        <is>
-          <t>iPeople PCS</t>
-        </is>
-      </c>
-      <c r="R83" t="inlineStr">
-        <is>
-          <t>PCS - iPeople</t>
-        </is>
-      </c>
-      <c r="S83" t="inlineStr">
-        <is>
-          <t>iPeople Nursing Assessment Forms</t>
         </is>
       </c>
     </row>
@@ -6852,7 +6852,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>HCA (Cloudera Kafka)-</t>
+          <t>HCA (Cloudera Kafka)-ADMO</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -6898,6 +6898,21 @@
       <c r="P85" t="inlineStr">
         <is>
           <t>Outbound</t>
+        </is>
+      </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>ADMO</t>
+        </is>
+      </c>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>ADT</t>
+        </is>
+      </c>
+      <c r="S85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admissions </t>
         </is>
       </c>
     </row>
@@ -6919,7 +6934,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>HCA (Cloudera Kafka)-</t>
+          <t>HCA (Cloudera Kafka)-CWSO</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -6965,6 +6980,21 @@
       <c r="P86" t="inlineStr">
         <is>
           <t>Outbound</t>
+        </is>
+      </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>CWSO</t>
+        </is>
+      </c>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>iPeople Scheduling</t>
+        </is>
+      </c>
+      <c r="S86" t="inlineStr">
+        <is>
+          <t>SIU</t>
         </is>
       </c>
     </row>
@@ -6986,7 +7016,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA (Cloudera Kafka)-Admissions </t>
+          <t>HCA (Cloudera Kafka)-CWSO</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -7036,17 +7066,17 @@
       </c>
       <c r="Q87" t="inlineStr">
         <is>
-          <t>ADMO</t>
+          <t>CWSO</t>
         </is>
       </c>
       <c r="R87" t="inlineStr">
         <is>
-          <t>ADT</t>
+          <t>SIU</t>
         </is>
       </c>
       <c r="S87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Admissions </t>
+          <t xml:space="preserve">Scheduling </t>
         </is>
       </c>
     </row>
@@ -7068,7 +7098,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA (Cloudera Kafka)-ITS DI Results </t>
+          <t>HCA (Cloudera Kafka)-IMMUN</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -7118,17 +7148,17 @@
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>ITSDIRO</t>
+          <t>IMMUN</t>
         </is>
       </c>
       <c r="R88" t="inlineStr">
         <is>
-          <t>ORU</t>
+          <t>VXU</t>
         </is>
       </c>
       <c r="S88" t="inlineStr">
         <is>
-          <t xml:space="preserve">ITS DI Results </t>
+          <t>MU-Immunizations</t>
         </is>
       </c>
     </row>
@@ -7150,7 +7180,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA (Cloudera Kafka)-ITS DI Results </t>
+          <t>HCA (Cloudera Kafka)-ITSDIRO</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -7232,7 +7262,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA (Cloudera Kafka)-ITS HM Results </t>
+          <t>HCA (Cloudera Kafka)-ITSDIRO</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -7282,7 +7312,7 @@
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>ITSHMRO</t>
+          <t>ITSDIRO</t>
         </is>
       </c>
       <c r="R90" t="inlineStr">
@@ -7292,7 +7322,7 @@
       </c>
       <c r="S90" t="inlineStr">
         <is>
-          <t xml:space="preserve">ITS HM Results </t>
+          <t xml:space="preserve">ITS DI Results </t>
         </is>
       </c>
     </row>
@@ -7314,7 +7344,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA (Cloudera Kafka)-Lab Results (Discrete) </t>
+          <t>HCA (Cloudera Kafka)-ITSHMRO</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -7364,7 +7394,7 @@
       </c>
       <c r="Q91" t="inlineStr">
         <is>
-          <t>LABRES</t>
+          <t>ITSHMRO</t>
         </is>
       </c>
       <c r="R91" t="inlineStr">
@@ -7374,7 +7404,7 @@
       </c>
       <c r="S91" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lab Results (Discrete) </t>
+          <t xml:space="preserve">ITS HM Results </t>
         </is>
       </c>
     </row>
@@ -7396,7 +7426,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA (Cloudera Kafka)-Lab Results (Discrete) </t>
+          <t>HCA (Cloudera Kafka)-LABRES</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -7478,7 +7508,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>HCA (Cloudera Kafka)-MU-Immunizations</t>
+          <t>HCA (Cloudera Kafka)-LABRES</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -7528,17 +7558,17 @@
       </c>
       <c r="Q93" t="inlineStr">
         <is>
-          <t>IMMUN</t>
+          <t>LABRES</t>
         </is>
       </c>
       <c r="R93" t="inlineStr">
         <is>
-          <t>VXU</t>
+          <t>ORU</t>
         </is>
       </c>
       <c r="S93" t="inlineStr">
         <is>
-          <t>MU-Immunizations</t>
+          <t xml:space="preserve">Lab Results (Discrete) </t>
         </is>
       </c>
     </row>
@@ -7560,7 +7590,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA (Cloudera Kafka)-OM Orders </t>
+          <t>HCA (Cloudera Kafka)-LABRES2</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -7610,17 +7640,17 @@
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t>OMORDO</t>
+          <t>LABRES2</t>
         </is>
       </c>
       <c r="R94" t="inlineStr">
         <is>
-          <t>iPeople OM Orders</t>
+          <t>ORU</t>
         </is>
       </c>
       <c r="S94" t="inlineStr">
         <is>
-          <t>ORM - iPeople</t>
+          <t>Pathology Results</t>
         </is>
       </c>
     </row>
@@ -7642,7 +7672,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>HCA (Cloudera Kafka)-Pathology Results</t>
+          <t>HCA (Cloudera Kafka)-LABRES2</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -7724,7 +7754,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>HCA (Cloudera Kafka)-Pathology Results</t>
+          <t>HCA (Cloudera Kafka)-OMORDO</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -7774,17 +7804,17 @@
       </c>
       <c r="Q96" t="inlineStr">
         <is>
-          <t>LABRES2</t>
+          <t>OMORDO</t>
         </is>
       </c>
       <c r="R96" t="inlineStr">
         <is>
-          <t>ORU</t>
+          <t>iPeople OM Orders</t>
         </is>
       </c>
       <c r="S96" t="inlineStr">
         <is>
-          <t>Pathology Results</t>
+          <t>ORM - iPeople</t>
         </is>
       </c>
     </row>
@@ -7806,7 +7836,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA (Cloudera Kafka)-Pharmacy Orders </t>
+          <t>HCA (Cloudera Kafka)-PHAORD</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -7888,7 +7918,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA (Cloudera Kafka)-Scheduling </t>
+          <t>HCA (Cloudera Kafka)-iPeople EDM</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -7938,17 +7968,17 @@
       </c>
       <c r="Q98" t="inlineStr">
         <is>
-          <t>CWSO</t>
+          <t>iPeople EDM</t>
         </is>
       </c>
       <c r="R98" t="inlineStr">
         <is>
-          <t>iPeople Scheduling</t>
+          <t>EDM - iPeople</t>
         </is>
       </c>
       <c r="S98" t="inlineStr">
         <is>
-          <t>SIU</t>
+          <t>iPeople ED Patient Visit Data</t>
         </is>
       </c>
     </row>
@@ -7970,7 +8000,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA (Cloudera Kafka)-Scheduling </t>
+          <t>HCA (Cloudera Kafka)-iPeople EDM</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -8020,17 +8050,17 @@
       </c>
       <c r="Q99" t="inlineStr">
         <is>
-          <t>CWSO</t>
+          <t>iPeople EDM</t>
         </is>
       </c>
       <c r="R99" t="inlineStr">
         <is>
-          <t>SIU</t>
+          <t>EDM - iPeople</t>
         </is>
       </c>
       <c r="S99" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scheduling </t>
+          <t>iPeople ED Patient Visit Data</t>
         </is>
       </c>
     </row>
@@ -8052,7 +8082,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>HCA (Cloudera Kafka)-iPeople ED Patient Visit Data</t>
+          <t>HCA (Cloudera Kafka)-iPeople Meds</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -8102,17 +8132,17 @@
       </c>
       <c r="Q100" t="inlineStr">
         <is>
-          <t>iPeople EDM</t>
+          <t>iPeople Meds</t>
         </is>
       </c>
       <c r="R100" t="inlineStr">
         <is>
-          <t>EDM - iPeople</t>
+          <t>RAS - iPeople</t>
         </is>
       </c>
       <c r="S100" t="inlineStr">
         <is>
-          <t>iPeople ED Patient Visit Data</t>
+          <t>iPeople Medication Administration</t>
         </is>
       </c>
     </row>
@@ -8134,7 +8164,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>HCA (Cloudera Kafka)-iPeople ED Patient Visit Data</t>
+          <t>HCA (Cloudera Kafka)-iPeople PCS</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -8184,17 +8214,17 @@
       </c>
       <c r="Q101" t="inlineStr">
         <is>
-          <t>iPeople EDM</t>
+          <t>iPeople PCS</t>
         </is>
       </c>
       <c r="R101" t="inlineStr">
         <is>
-          <t>EDM - iPeople</t>
+          <t>PCS - iPeople</t>
         </is>
       </c>
       <c r="S101" t="inlineStr">
         <is>
-          <t>iPeople ED Patient Visit Data</t>
+          <t>iPeople Nursing Assessment Forms</t>
         </is>
       </c>
     </row>
@@ -8216,7 +8246,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>HCA (Cloudera Kafka)-iPeople Medication Administration</t>
+          <t>HCA (Cloudera Kafka)-iPeople PCS</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
@@ -8266,17 +8296,17 @@
       </c>
       <c r="Q102" t="inlineStr">
         <is>
-          <t>iPeople Meds</t>
+          <t>iPeople PCS</t>
         </is>
       </c>
       <c r="R102" t="inlineStr">
         <is>
-          <t>RAS - iPeople</t>
+          <t>PCS - iPeople</t>
         </is>
       </c>
       <c r="S102" t="inlineStr">
         <is>
-          <t>iPeople Medication Administration</t>
+          <t>iPeople Nursing Assessment Forms</t>
         </is>
       </c>
     </row>
@@ -8298,7 +8328,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>HCA (Cloudera Kafka)-iPeople Nursing Assessment Forms</t>
+          <t>HCA (Cloudera Kafka)-radord</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -8344,21 +8374,6 @@
       <c r="P103" t="inlineStr">
         <is>
           <t>Outbound</t>
-        </is>
-      </c>
-      <c r="Q103" t="inlineStr">
-        <is>
-          <t>iPeople PCS</t>
-        </is>
-      </c>
-      <c r="R103" t="inlineStr">
-        <is>
-          <t>PCS - iPeople</t>
-        </is>
-      </c>
-      <c r="S103" t="inlineStr">
-        <is>
-          <t>iPeople Nursing Assessment Forms</t>
         </is>
       </c>
     </row>
@@ -8380,7 +8395,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>HCA (Cloudera Kafka)-iPeople Nursing Assessment Forms</t>
+          <t>HCA (Cloudera Kafka)-radord</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
@@ -8426,21 +8441,6 @@
       <c r="P104" t="inlineStr">
         <is>
           <t>Outbound</t>
-        </is>
-      </c>
-      <c r="Q104" t="inlineStr">
-        <is>
-          <t>iPeople PCS</t>
-        </is>
-      </c>
-      <c r="R104" t="inlineStr">
-        <is>
-          <t>PCS - iPeople</t>
-        </is>
-      </c>
-      <c r="S104" t="inlineStr">
-        <is>
-          <t>iPeople Nursing Assessment Forms</t>
         </is>
       </c>
     </row>
@@ -8524,7 +8524,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA (EDW CDM)-Scheduling </t>
+          <t>HCA (EDW CDM)-CWSO</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
@@ -8668,7 +8668,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA (Revive)-ITS HM Results </t>
+          <t>HCA (Revive)-ITSHMRO</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>HCA (SMART to Optiflex)-</t>
+          <t>HCA (SMART to Optiflex)-multi</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
@@ -8941,7 +8941,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>HCA (SMART)-</t>
+          <t>HCA (SMART)-ADMO</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
@@ -8986,7 +8986,22 @@
       </c>
       <c r="P112" t="inlineStr">
         <is>
-          <t>Inbound</t>
+          <t>Outbound</t>
+        </is>
+      </c>
+      <c r="Q112" t="inlineStr">
+        <is>
+          <t>ADMO</t>
+        </is>
+      </c>
+      <c r="R112" t="inlineStr">
+        <is>
+          <t>ADT</t>
+        </is>
+      </c>
+      <c r="S112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admissions </t>
         </is>
       </c>
     </row>
@@ -9008,7 +9023,7 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>HCA (SMART)-</t>
+          <t>HCA (SMART)-multi</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
@@ -9075,7 +9090,7 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA (SMART)-Admissions </t>
+          <t>HCA (SMART)-multi</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
@@ -9120,22 +9135,7 @@
       </c>
       <c r="P114" t="inlineStr">
         <is>
-          <t>Outbound</t>
-        </is>
-      </c>
-      <c r="Q114" t="inlineStr">
-        <is>
-          <t>ADMO</t>
-        </is>
-      </c>
-      <c r="R114" t="inlineStr">
-        <is>
-          <t>ADT</t>
-        </is>
-      </c>
-      <c r="S114" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Admissions </t>
+          <t>Inbound</t>
         </is>
       </c>
     </row>
@@ -9219,7 +9219,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA D&amp;IS (EIS Biztalk Platform to UDS PROi)-ITS HM Results </t>
+          <t>HCA D&amp;IS (EIS Biztalk Platform to UDS PROi)-ITSHMRO</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
@@ -9363,7 +9363,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>HCA D&amp;IS (EIS Biztalk Platform)-</t>
+          <t>HCA D&amp;IS (EIS Biztalk Platform)-ADMO</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
@@ -9409,6 +9409,21 @@
       <c r="P118" t="inlineStr">
         <is>
           <t>Outbound</t>
+        </is>
+      </c>
+      <c r="Q118" t="inlineStr">
+        <is>
+          <t>ADMO</t>
+        </is>
+      </c>
+      <c r="R118" t="inlineStr">
+        <is>
+          <t>ADT</t>
+        </is>
+      </c>
+      <c r="S118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admissions </t>
         </is>
       </c>
     </row>
@@ -9430,7 +9445,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA D&amp;IS (EIS Biztalk Platform)-Admissions </t>
+          <t>HCA D&amp;IS (EIS Biztalk Platform)-CWSO</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
@@ -9480,17 +9495,17 @@
       </c>
       <c r="Q119" t="inlineStr">
         <is>
-          <t>ADMO</t>
+          <t>CWSO</t>
         </is>
       </c>
       <c r="R119" t="inlineStr">
         <is>
-          <t>ADT</t>
+          <t>iPeople Scheduling</t>
         </is>
       </c>
       <c r="S119" t="inlineStr">
         <is>
-          <t xml:space="preserve">Admissions </t>
+          <t>SIU</t>
         </is>
       </c>
     </row>
@@ -9512,7 +9527,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA D&amp;IS (EIS Biztalk Platform)-ITS DI Results </t>
+          <t>HCA D&amp;IS (EIS Biztalk Platform)-CWSO</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -9562,17 +9577,17 @@
       </c>
       <c r="Q120" t="inlineStr">
         <is>
-          <t>ITSDIRO</t>
+          <t>CWSO</t>
         </is>
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>ORU</t>
+          <t>SIU</t>
         </is>
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t xml:space="preserve">ITS DI Results </t>
+          <t xml:space="preserve">Scheduling </t>
         </is>
       </c>
     </row>
@@ -9594,7 +9609,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA D&amp;IS (EIS Biztalk Platform)-ITS HM Results </t>
+          <t>HCA D&amp;IS (EIS Biztalk Platform)-IMMUN</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
@@ -9644,17 +9659,17 @@
       </c>
       <c r="Q121" t="inlineStr">
         <is>
-          <t>ITSHMRO</t>
+          <t>IMMUN</t>
         </is>
       </c>
       <c r="R121" t="inlineStr">
         <is>
-          <t>ORU</t>
+          <t>VXU</t>
         </is>
       </c>
       <c r="S121" t="inlineStr">
         <is>
-          <t xml:space="preserve">ITS HM Results </t>
+          <t>MU-Immunizations</t>
         </is>
       </c>
     </row>
@@ -9676,7 +9691,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA D&amp;IS (EIS Biztalk Platform)-Lab Results (Discrete) </t>
+          <t>HCA D&amp;IS (EIS Biztalk Platform)-ITSDIRO</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
@@ -9726,7 +9741,7 @@
       </c>
       <c r="Q122" t="inlineStr">
         <is>
-          <t>LABRES</t>
+          <t>ITSDIRO</t>
         </is>
       </c>
       <c r="R122" t="inlineStr">
@@ -9736,7 +9751,7 @@
       </c>
       <c r="S122" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lab Results (Discrete) </t>
+          <t xml:space="preserve">ITS DI Results </t>
         </is>
       </c>
     </row>
@@ -9758,7 +9773,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>HCA D&amp;IS (EIS Biztalk Platform)-MU-Electronic Lab Reporting</t>
+          <t>HCA D&amp;IS (EIS Biztalk Platform)-ITSHMRO</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
@@ -9808,7 +9823,7 @@
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t>PHELR</t>
+          <t>ITSHMRO</t>
         </is>
       </c>
       <c r="R123" t="inlineStr">
@@ -9818,7 +9833,7 @@
       </c>
       <c r="S123" t="inlineStr">
         <is>
-          <t>MU-Electronic Lab Reporting</t>
+          <t xml:space="preserve">ITS HM Results </t>
         </is>
       </c>
     </row>
@@ -9840,7 +9855,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>HCA D&amp;IS (EIS Biztalk Platform)-MU-Immunizations</t>
+          <t>HCA D&amp;IS (EIS Biztalk Platform)-LABRES</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
@@ -9890,17 +9905,17 @@
       </c>
       <c r="Q124" t="inlineStr">
         <is>
-          <t>IMMUN</t>
+          <t>LABRES</t>
         </is>
       </c>
       <c r="R124" t="inlineStr">
         <is>
-          <t>VXU</t>
+          <t>ORU</t>
         </is>
       </c>
       <c r="S124" t="inlineStr">
         <is>
-          <t>MU-Immunizations</t>
+          <t xml:space="preserve">Lab Results (Discrete) </t>
         </is>
       </c>
     </row>
@@ -9922,7 +9937,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>HCA D&amp;IS (EIS Biztalk Platform)-MU-Syndromic Surveillance</t>
+          <t>HCA D&amp;IS (EIS Biztalk Platform)-LABRES2</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
@@ -9972,17 +9987,17 @@
       </c>
       <c r="Q125" t="inlineStr">
         <is>
-          <t>PHSS</t>
+          <t>LABRES2</t>
         </is>
       </c>
       <c r="R125" t="inlineStr">
         <is>
-          <t>ADT</t>
+          <t>ORU</t>
         </is>
       </c>
       <c r="S125" t="inlineStr">
         <is>
-          <t>MU-Syndromic Surveillance</t>
+          <t>Pathology Results</t>
         </is>
       </c>
     </row>
@@ -10004,7 +10019,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA D&amp;IS (EIS Biztalk Platform)-OM Orders </t>
+          <t>HCA D&amp;IS (EIS Biztalk Platform)-OMORDO</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
@@ -10086,7 +10101,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA D&amp;IS (EIS Biztalk Platform)-OM Orders </t>
+          <t>HCA D&amp;IS (EIS Biztalk Platform)-OMORDO</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
@@ -10168,7 +10183,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>HCA D&amp;IS (EIS Biztalk Platform)-Pathology Results</t>
+          <t>HCA D&amp;IS (EIS Biztalk Platform)-PHAORD</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
@@ -10218,17 +10233,17 @@
       </c>
       <c r="Q128" t="inlineStr">
         <is>
-          <t>LABRES2</t>
+          <t>PHAORD</t>
         </is>
       </c>
       <c r="R128" t="inlineStr">
         <is>
-          <t>ORU</t>
+          <t>RDE</t>
         </is>
       </c>
       <c r="S128" t="inlineStr">
         <is>
-          <t>Pathology Results</t>
+          <t xml:space="preserve">Pharmacy Orders </t>
         </is>
       </c>
     </row>
@@ -10250,7 +10265,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA D&amp;IS (EIS Biztalk Platform)-Pharmacy Orders </t>
+          <t>HCA D&amp;IS (EIS Biztalk Platform)-PHELR</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
@@ -10300,17 +10315,17 @@
       </c>
       <c r="Q129" t="inlineStr">
         <is>
-          <t>PHAORD</t>
+          <t>PHELR</t>
         </is>
       </c>
       <c r="R129" t="inlineStr">
         <is>
-          <t>RDE</t>
+          <t>ORU</t>
         </is>
       </c>
       <c r="S129" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pharmacy Orders </t>
+          <t>MU-Electronic Lab Reporting</t>
         </is>
       </c>
     </row>
@@ -10332,7 +10347,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA D&amp;IS (EIS Biztalk Platform)-Scheduling </t>
+          <t>HCA D&amp;IS (EIS Biztalk Platform)-PHSS</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
@@ -10382,17 +10397,17 @@
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>CWSO</t>
+          <t>PHSS</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
         <is>
-          <t>iPeople Scheduling</t>
+          <t>ADT</t>
         </is>
       </c>
       <c r="S130" t="inlineStr">
         <is>
-          <t>SIU</t>
+          <t>MU-Syndromic Surveillance</t>
         </is>
       </c>
     </row>
@@ -10414,7 +10429,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA D&amp;IS (EIS Biztalk Platform)-Scheduling </t>
+          <t>HCA D&amp;IS (EIS Biztalk Platform)-iPeople EDM</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
@@ -10464,17 +10479,17 @@
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>CWSO</t>
+          <t>iPeople EDM</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
         <is>
-          <t>SIU</t>
+          <t>EDM - iPeople</t>
         </is>
       </c>
       <c r="S131" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scheduling </t>
+          <t>iPeople ED Patient Visit Data</t>
         </is>
       </c>
     </row>
@@ -10496,7 +10511,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>HCA D&amp;IS (EIS Biztalk Platform)-iPeople ED Patient Visit Data</t>
+          <t>HCA D&amp;IS (EIS Biztalk Platform)-iPeople Meds</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
@@ -10546,17 +10561,17 @@
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>iPeople EDM</t>
+          <t>iPeople Meds</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">
         <is>
-          <t>EDM - iPeople</t>
+          <t>RAS - iPeople</t>
         </is>
       </c>
       <c r="S132" t="inlineStr">
         <is>
-          <t>iPeople ED Patient Visit Data</t>
+          <t>iPeople Medication Administration</t>
         </is>
       </c>
     </row>
@@ -10578,7 +10593,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>HCA D&amp;IS (EIS Biztalk Platform)-iPeople Medication Administration</t>
+          <t>HCA D&amp;IS (EIS Biztalk Platform)-iPeople PCS</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
@@ -10628,17 +10643,17 @@
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>iPeople Meds</t>
+          <t>iPeople PCS</t>
         </is>
       </c>
       <c r="R133" t="inlineStr">
         <is>
-          <t>RAS - iPeople</t>
+          <t>PCS - iPeople</t>
         </is>
       </c>
       <c r="S133" t="inlineStr">
         <is>
-          <t>iPeople Medication Administration</t>
+          <t>iPeople Nursing Assessment Forms</t>
         </is>
       </c>
     </row>
@@ -10660,7 +10675,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>HCA D&amp;IS (EIS Biztalk Platform)-iPeople Nursing Assessment Forms</t>
+          <t>HCA D&amp;IS (EIS Biztalk Platform)-radord</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
@@ -10706,21 +10721,6 @@
       <c r="P134" t="inlineStr">
         <is>
           <t>Outbound</t>
-        </is>
-      </c>
-      <c r="Q134" t="inlineStr">
-        <is>
-          <t>iPeople PCS</t>
-        </is>
-      </c>
-      <c r="R134" t="inlineStr">
-        <is>
-          <t>PCS - iPeople</t>
-        </is>
-      </c>
-      <c r="S134" t="inlineStr">
-        <is>
-          <t>iPeople Nursing Assessment Forms</t>
         </is>
       </c>
     </row>
@@ -10804,7 +10804,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA D&amp;IS (FHIR Web Services)-Admissions </t>
+          <t>HCA D&amp;IS (FHIR Web Services)-ADMO</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
@@ -10886,7 +10886,7 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA D&amp;IS (FHIR Web Services)-Admissions </t>
+          <t>HCA D&amp;IS (FHIR Web Services)-ADMO</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
@@ -11030,7 +11030,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA D&amp;IS (HCA 5.6)-ITS HM Results </t>
+          <t>HCA D&amp;IS (HCA 5.6)-ITSHMRO</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
@@ -11174,7 +11174,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>HCA D&amp;IS (MPF-Patient Folder/HPF Facility)-</t>
+          <t>HCA D&amp;IS (MPF-Patient Folder/HPF Facility)-imgurl</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
@@ -11303,7 +11303,7 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>HCA D&amp;IS (Null-Terminates Message)-</t>
+          <t>HCA D&amp;IS (Null-Terminates Message)-iti08</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
@@ -11432,7 +11432,7 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>HCA D&amp;IS (Waterpark to UDS PROi)-</t>
+          <t>HCA D&amp;IS (Waterpark to UDS PROi)-irfpai</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
@@ -11561,7 +11561,7 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>HCA D&amp;IS (Waterpark)-</t>
+          <t>HCA D&amp;IS (Waterpark)-ADMO</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
@@ -11607,6 +11607,21 @@
       <c r="P147" t="inlineStr">
         <is>
           <t>Outbound</t>
+        </is>
+      </c>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>ADMO</t>
+        </is>
+      </c>
+      <c r="R147" t="inlineStr">
+        <is>
+          <t>ADT</t>
+        </is>
+      </c>
+      <c r="S147" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admissions </t>
         </is>
       </c>
     </row>
@@ -11628,7 +11643,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA D&amp;IS (Waterpark)-Admissions </t>
+          <t>HCA D&amp;IS (Waterpark)-CWSO</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
@@ -11678,17 +11693,17 @@
       </c>
       <c r="Q148" t="inlineStr">
         <is>
-          <t>ADMO</t>
+          <t>CWSO</t>
         </is>
       </c>
       <c r="R148" t="inlineStr">
         <is>
-          <t>ADT</t>
+          <t>iPeople Scheduling</t>
         </is>
       </c>
       <c r="S148" t="inlineStr">
         <is>
-          <t xml:space="preserve">Admissions </t>
+          <t>SIU</t>
         </is>
       </c>
     </row>
@@ -11710,7 +11725,7 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA D&amp;IS (Waterpark)-ITS DI Results </t>
+          <t>HCA D&amp;IS (Waterpark)-CWSO</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
@@ -11760,17 +11775,17 @@
       </c>
       <c r="Q149" t="inlineStr">
         <is>
-          <t>ITSDIRO</t>
+          <t>CWSO</t>
         </is>
       </c>
       <c r="R149" t="inlineStr">
         <is>
-          <t>ORU</t>
+          <t>SIU</t>
         </is>
       </c>
       <c r="S149" t="inlineStr">
         <is>
-          <t xml:space="preserve">ITS DI Results </t>
+          <t xml:space="preserve">Scheduling </t>
         </is>
       </c>
     </row>
@@ -11792,7 +11807,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA D&amp;IS (Waterpark)-ITS HM Results </t>
+          <t>HCA D&amp;IS (Waterpark)-IMMUN</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
@@ -11842,17 +11857,17 @@
       </c>
       <c r="Q150" t="inlineStr">
         <is>
-          <t>ITSHMRO</t>
+          <t>IMMUN</t>
         </is>
       </c>
       <c r="R150" t="inlineStr">
         <is>
-          <t>ORU</t>
+          <t>VXU</t>
         </is>
       </c>
       <c r="S150" t="inlineStr">
         <is>
-          <t xml:space="preserve">ITS HM Results </t>
+          <t>MU-Immunizations</t>
         </is>
       </c>
     </row>
@@ -11874,7 +11889,7 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>HCA D&amp;IS (Waterpark)-Immunization Query</t>
+          <t>HCA D&amp;IS (Waterpark)-IMMUNQRY</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
@@ -11956,7 +11971,7 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA D&amp;IS (Waterpark)-Lab Results (Discrete) </t>
+          <t>HCA D&amp;IS (Waterpark)-ITSDIRO</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
@@ -12006,7 +12021,7 @@
       </c>
       <c r="Q152" t="inlineStr">
         <is>
-          <t>LABRES</t>
+          <t>ITSDIRO</t>
         </is>
       </c>
       <c r="R152" t="inlineStr">
@@ -12016,7 +12031,7 @@
       </c>
       <c r="S152" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lab Results (Discrete) </t>
+          <t xml:space="preserve">ITS DI Results </t>
         </is>
       </c>
     </row>
@@ -12038,7 +12053,7 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>HCA D&amp;IS (Waterpark)-MU-Immunizations</t>
+          <t>HCA D&amp;IS (Waterpark)-ITSHMRO</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
@@ -12088,17 +12103,17 @@
       </c>
       <c r="Q153" t="inlineStr">
         <is>
-          <t>IMMUN</t>
+          <t>ITSHMRO</t>
         </is>
       </c>
       <c r="R153" t="inlineStr">
         <is>
-          <t>VXU</t>
+          <t>ORU</t>
         </is>
       </c>
       <c r="S153" t="inlineStr">
         <is>
-          <t>MU-Immunizations</t>
+          <t xml:space="preserve">ITS HM Results </t>
         </is>
       </c>
     </row>
@@ -12120,7 +12135,7 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>HCA D&amp;IS (Waterpark)-MU-Syndromic Surveillance</t>
+          <t>HCA D&amp;IS (Waterpark)-LABRES</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
@@ -12170,17 +12185,17 @@
       </c>
       <c r="Q154" t="inlineStr">
         <is>
-          <t>PHSS</t>
+          <t>LABRES</t>
         </is>
       </c>
       <c r="R154" t="inlineStr">
         <is>
-          <t>ADT</t>
+          <t>ORU</t>
         </is>
       </c>
       <c r="S154" t="inlineStr">
         <is>
-          <t>MU-Syndromic Surveillance</t>
+          <t xml:space="preserve">Lab Results (Discrete) </t>
         </is>
       </c>
     </row>
@@ -12202,7 +12217,7 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA D&amp;IS (Waterpark)-OM Orders </t>
+          <t>HCA D&amp;IS (Waterpark)-LABRES2</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
@@ -12252,17 +12267,17 @@
       </c>
       <c r="Q155" t="inlineStr">
         <is>
-          <t>OMORDO</t>
+          <t>LABRES2</t>
         </is>
       </c>
       <c r="R155" t="inlineStr">
         <is>
-          <t>iPeople OM Orders</t>
+          <t>ORU</t>
         </is>
       </c>
       <c r="S155" t="inlineStr">
         <is>
-          <t>ORM - iPeople</t>
+          <t>Pathology Results</t>
         </is>
       </c>
     </row>
@@ -12284,7 +12299,7 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA D&amp;IS (Waterpark)-OM Orders </t>
+          <t>HCA D&amp;IS (Waterpark)-OMORDO</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
@@ -12339,12 +12354,12 @@
       </c>
       <c r="R156" t="inlineStr">
         <is>
-          <t>ORM</t>
+          <t>iPeople OM Orders</t>
         </is>
       </c>
       <c r="S156" t="inlineStr">
         <is>
-          <t xml:space="preserve">OM Orders </t>
+          <t>ORM - iPeople</t>
         </is>
       </c>
     </row>
@@ -12366,7 +12381,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>HCA D&amp;IS (Waterpark)-Pathology Results</t>
+          <t>HCA D&amp;IS (Waterpark)-OMORDO</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
@@ -12416,17 +12431,17 @@
       </c>
       <c r="Q157" t="inlineStr">
         <is>
-          <t>LABRES2</t>
+          <t>OMORDO</t>
         </is>
       </c>
       <c r="R157" t="inlineStr">
         <is>
-          <t>ORU</t>
+          <t>ORM</t>
         </is>
       </c>
       <c r="S157" t="inlineStr">
         <is>
-          <t>Pathology Results</t>
+          <t xml:space="preserve">OM Orders </t>
         </is>
       </c>
     </row>
@@ -12448,7 +12463,7 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA D&amp;IS (Waterpark)-Pharmacy Orders </t>
+          <t>HCA D&amp;IS (Waterpark)-PHAORD</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
@@ -12530,7 +12545,7 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA D&amp;IS (Waterpark)-Scheduling </t>
+          <t>HCA D&amp;IS (Waterpark)-PHSS</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
@@ -12580,17 +12595,17 @@
       </c>
       <c r="Q159" t="inlineStr">
         <is>
-          <t>CWSO</t>
+          <t>PHSS</t>
         </is>
       </c>
       <c r="R159" t="inlineStr">
         <is>
-          <t>iPeople Scheduling</t>
+          <t>ADT</t>
         </is>
       </c>
       <c r="S159" t="inlineStr">
         <is>
-          <t>SIU</t>
+          <t>MU-Syndromic Surveillance</t>
         </is>
       </c>
     </row>
@@ -12612,7 +12627,7 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA D&amp;IS (Waterpark)-Scheduling </t>
+          <t>HCA D&amp;IS (Waterpark)-iPeople EDM</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
@@ -12662,17 +12677,17 @@
       </c>
       <c r="Q160" t="inlineStr">
         <is>
-          <t>CWSO</t>
+          <t>iPeople EDM</t>
         </is>
       </c>
       <c r="R160" t="inlineStr">
         <is>
-          <t>SIU</t>
+          <t>EDM - iPeople</t>
         </is>
       </c>
       <c r="S160" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scheduling </t>
+          <t>iPeople ED Patient Visit Data</t>
         </is>
       </c>
     </row>
@@ -12694,7 +12709,7 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>HCA D&amp;IS (Waterpark)-iPeople ED Patient Visit Data</t>
+          <t>HCA D&amp;IS (Waterpark)-iPeople Meds</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
@@ -12744,17 +12759,17 @@
       </c>
       <c r="Q161" t="inlineStr">
         <is>
-          <t>iPeople EDM</t>
+          <t>iPeople Meds</t>
         </is>
       </c>
       <c r="R161" t="inlineStr">
         <is>
-          <t>EDM - iPeople</t>
+          <t>RAS - iPeople</t>
         </is>
       </c>
       <c r="S161" t="inlineStr">
         <is>
-          <t>iPeople ED Patient Visit Data</t>
+          <t>iPeople Medication Administration</t>
         </is>
       </c>
     </row>
@@ -12776,7 +12791,7 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>HCA D&amp;IS (Waterpark)-iPeople Medication Administration</t>
+          <t>HCA D&amp;IS (Waterpark)-iPeople PCS</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
@@ -12826,17 +12841,17 @@
       </c>
       <c r="Q162" t="inlineStr">
         <is>
-          <t>iPeople Meds</t>
+          <t>iPeople PCS</t>
         </is>
       </c>
       <c r="R162" t="inlineStr">
         <is>
-          <t>RAS - iPeople</t>
+          <t>PCS - iPeople</t>
         </is>
       </c>
       <c r="S162" t="inlineStr">
         <is>
-          <t>iPeople Medication Administration</t>
+          <t>iPeople Nursing Assessment Forms</t>
         </is>
       </c>
     </row>
@@ -12858,7 +12873,7 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>HCA D&amp;IS (Waterpark)-iPeople Nursing Assessment Forms</t>
+          <t>HCA D&amp;IS (Waterpark)-radord</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
@@ -12904,21 +12919,6 @@
       <c r="P163" t="inlineStr">
         <is>
           <t>Outbound</t>
-        </is>
-      </c>
-      <c r="Q163" t="inlineStr">
-        <is>
-          <t>iPeople PCS</t>
-        </is>
-      </c>
-      <c r="R163" t="inlineStr">
-        <is>
-          <t>PCS - iPeople</t>
-        </is>
-      </c>
-      <c r="S163" t="inlineStr">
-        <is>
-          <t>iPeople Nursing Assessment Forms</t>
         </is>
       </c>
     </row>
@@ -13002,7 +13002,7 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA Parallon (Charge Master)-SMART Procedure Codes </t>
+          <t>HCA Parallon (Charge Master)-MISPROC</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
@@ -13146,7 +13146,7 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t xml:space="preserve">HCA Parallon (eCapture)-Admissions </t>
+          <t>HCA Parallon (eCapture)-ADMO</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
@@ -13290,7 +13290,7 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t xml:space="preserve">Health Catalyst (HCare Hub)-Admissions </t>
+          <t>Health Catalyst (HCare Hub)-ADMO</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
@@ -13372,7 +13372,7 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t xml:space="preserve">Health Catalyst (HCare Hub)-ITS DI Results </t>
+          <t>Health Catalyst (HCare Hub)-ITSDIRO</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
@@ -13454,7 +13454,7 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t xml:space="preserve">Health Catalyst (HCare Hub)-ITS HM Results </t>
+          <t>Health Catalyst (HCare Hub)-ITSHMRO</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
@@ -13536,7 +13536,7 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t xml:space="preserve">Health Catalyst (HCare Hub)-Lab Results (Discrete) </t>
+          <t>Health Catalyst (HCare Hub)-LABRES</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
@@ -13618,7 +13618,7 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>Health Catalyst (HCare Hub)-Pathology Results</t>
+          <t>Health Catalyst (HCare Hub)-LABRES2</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
@@ -13762,7 +13762,7 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hill-Rom (Navacare Patient Flow)-Admissions </t>
+          <t>Hill-Rom (Navacare Patient Flow)-ADMO</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
@@ -13906,7 +13906,7 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hill-Rom/Welch Allyn (Connex CS)-Admissions </t>
+          <t>Hill-Rom/Welch Allyn (Connex CS)-ADMO</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
@@ -13988,7 +13988,7 @@
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hill-Rom/Welch Allyn (Connex CS)-Clinical Monitoring Results </t>
+          <t>Hill-Rom/Welch Allyn (Connex CS)-PCSCMI</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
@@ -14132,7 +14132,7 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hospira (Theradoc)-Admissions </t>
+          <t>Hospira (Theradoc)-ADMO</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
@@ -14214,7 +14214,7 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hospira (Theradoc)-ITS DI Results </t>
+          <t>Hospira (Theradoc)-ITSDIRO</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
@@ -14296,7 +14296,7 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hospira (Theradoc)-ITS HM Results </t>
+          <t>Hospira (Theradoc)-ITSHMRO</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
@@ -14378,7 +14378,7 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hospira (Theradoc)-Lab Results (Discrete) </t>
+          <t>Hospira (Theradoc)-LABRES</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
@@ -14460,7 +14460,7 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hospira (Theradoc)-OM Orders </t>
+          <t>Hospira (Theradoc)-OMORDO</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
@@ -14542,7 +14542,7 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hospira (Theradoc)-Pharmacy Orders </t>
+          <t>Hospira (Theradoc)-PHAORD</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
@@ -14624,7 +14624,7 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>Hospira (Theradoc)-iPeople ED Patient Visit Data</t>
+          <t>Hospira (Theradoc)-iPeople EDM</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
@@ -14706,7 +14706,7 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>Hospira (Theradoc)-iPeople Medication Administration</t>
+          <t>Hospira (Theradoc)-iPeople Meds</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
@@ -14788,7 +14788,7 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>Hospira (Theradoc)-iPeople Nursing Assessment Forms</t>
+          <t>Hospira (Theradoc)-iPeople PCS</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
@@ -14932,7 +14932,7 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hyland (Onbase RX-ADT/Link Orders)-Admissions </t>
+          <t>Hyland (Onbase RX-ADT/Link Orders)-ADMO</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
@@ -15076,7 +15076,7 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>Hyland (Onbase to MPF-Patient Folder/HPF Facility)-</t>
+          <t>Hyland (Onbase to MPF-Patient Folder/HPF Facility)-imgurl</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
@@ -15205,7 +15205,7 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hyland (Onbase)-Admissions </t>
+          <t>Hyland (Onbase)-ADMO</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
@@ -15349,7 +15349,7 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t xml:space="preserve">IBM (Consent Management)-Admissions </t>
+          <t>IBM (Consent Management)-ADMO</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
@@ -15493,7 +15493,7 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t xml:space="preserve">IMS Integrated Medical Systems (ReadyTracker-Tissue)-Admissions </t>
+          <t>IMS Integrated Medical Systems (ReadyTracker-Tissue)-ADMO</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
@@ -15575,7 +15575,7 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t xml:space="preserve">IMS Integrated Medical Systems (ReadyTracker-Tissue)-Tissue Tracking </t>
+          <t>IMS Integrated Medical Systems (ReadyTracker-Tissue)-SURTSD</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
@@ -15719,7 +15719,7 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t xml:space="preserve">Initiate (Initiate)-Admissions </t>
+          <t>Initiate (Initiate)-ADMO</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
@@ -15801,7 +15801,7 @@
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t xml:space="preserve">Initiate (Initiate)-Admissions </t>
+          <t>Initiate (Initiate)-ADMO</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
@@ -15945,7 +15945,7 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>Iodine Software (Iodine-Facility)-</t>
+          <t>Iodine Software (Iodine-Facility)-ADMO</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
@@ -15991,6 +15991,21 @@
       <c r="P204" t="inlineStr">
         <is>
           <t>Outbound</t>
+        </is>
+      </c>
+      <c r="Q204" t="inlineStr">
+        <is>
+          <t>ADMO</t>
+        </is>
+      </c>
+      <c r="R204" t="inlineStr">
+        <is>
+          <t>ADT</t>
+        </is>
+      </c>
+      <c r="S204" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admissions </t>
         </is>
       </c>
     </row>
@@ -16012,7 +16027,7 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t xml:space="preserve">Iodine Software (Iodine-Facility)-Admissions </t>
+          <t>Iodine Software (Iodine-Facility)-ITSDIRO</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
@@ -16062,17 +16077,17 @@
       </c>
       <c r="Q205" t="inlineStr">
         <is>
-          <t>ADMO</t>
+          <t>ITSDIRO</t>
         </is>
       </c>
       <c r="R205" t="inlineStr">
         <is>
-          <t>ADT</t>
+          <t>ORU</t>
         </is>
       </c>
       <c r="S205" t="inlineStr">
         <is>
-          <t xml:space="preserve">Admissions </t>
+          <t xml:space="preserve">ITS DI Results </t>
         </is>
       </c>
     </row>
@@ -16094,7 +16109,7 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t xml:space="preserve">Iodine Software (Iodine-Facility)-ITS DI Results </t>
+          <t>Iodine Software (Iodine-Facility)-ITSHMRO</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
@@ -16144,7 +16159,7 @@
       </c>
       <c r="Q206" t="inlineStr">
         <is>
-          <t>ITSDIRO</t>
+          <t>ITSHMRO</t>
         </is>
       </c>
       <c r="R206" t="inlineStr">
@@ -16154,7 +16169,7 @@
       </c>
       <c r="S206" t="inlineStr">
         <is>
-          <t xml:space="preserve">ITS DI Results </t>
+          <t xml:space="preserve">ITS HM Results </t>
         </is>
       </c>
     </row>
@@ -16176,7 +16191,7 @@
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t xml:space="preserve">Iodine Software (Iodine-Facility)-ITS HM Results </t>
+          <t>Iodine Software (Iodine-Facility)-LABRES</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
@@ -16226,7 +16241,7 @@
       </c>
       <c r="Q207" t="inlineStr">
         <is>
-          <t>ITSHMRO</t>
+          <t>LABRES</t>
         </is>
       </c>
       <c r="R207" t="inlineStr">
@@ -16236,7 +16251,7 @@
       </c>
       <c r="S207" t="inlineStr">
         <is>
-          <t xml:space="preserve">ITS HM Results </t>
+          <t xml:space="preserve">Lab Results (Discrete) </t>
         </is>
       </c>
     </row>
@@ -16258,7 +16273,7 @@
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t xml:space="preserve">Iodine Software (Iodine-Facility)-Lab Results (Discrete) </t>
+          <t>Iodine Software (Iodine-Facility)-LABRES2</t>
         </is>
       </c>
       <c r="H208" t="inlineStr">
@@ -16308,7 +16323,7 @@
       </c>
       <c r="Q208" t="inlineStr">
         <is>
-          <t>LABRES</t>
+          <t>LABRES2</t>
         </is>
       </c>
       <c r="R208" t="inlineStr">
@@ -16318,7 +16333,7 @@
       </c>
       <c r="S208" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lab Results (Discrete) </t>
+          <t>Pathology Results</t>
         </is>
       </c>
     </row>
@@ -16340,7 +16355,7 @@
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t xml:space="preserve">Iodine Software (Iodine-Facility)-OM Orders </t>
+          <t>Iodine Software (Iodine-Facility)-OMORDO</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
@@ -16422,7 +16437,7 @@
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>Iodine Software (Iodine-Facility)-Pathology Results</t>
+          <t>Iodine Software (Iodine-Facility)-PHAORD</t>
         </is>
       </c>
       <c r="H210" t="inlineStr">
@@ -16472,17 +16487,17 @@
       </c>
       <c r="Q210" t="inlineStr">
         <is>
-          <t>LABRES2</t>
+          <t>PHAORD</t>
         </is>
       </c>
       <c r="R210" t="inlineStr">
         <is>
-          <t>ORU</t>
+          <t>RDE</t>
         </is>
       </c>
       <c r="S210" t="inlineStr">
         <is>
-          <t>Pathology Results</t>
+          <t xml:space="preserve">Pharmacy Orders </t>
         </is>
       </c>
     </row>
@@ -16504,7 +16519,7 @@
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t xml:space="preserve">Iodine Software (Iodine-Facility)-Pharmacy Orders </t>
+          <t>Iodine Software (Iodine-Facility)-radord</t>
         </is>
       </c>
       <c r="H211" t="inlineStr">
@@ -16550,21 +16565,6 @@
       <c r="P211" t="inlineStr">
         <is>
           <t>Outbound</t>
-        </is>
-      </c>
-      <c r="Q211" t="inlineStr">
-        <is>
-          <t>PHAORD</t>
-        </is>
-      </c>
-      <c r="R211" t="inlineStr">
-        <is>
-          <t>RDE</t>
-        </is>
-      </c>
-      <c r="S211" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pharmacy Orders </t>
         </is>
       </c>
     </row>
@@ -16648,7 +16648,7 @@
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t xml:space="preserve">MSN Healthcare Solutions (Intellirad)-Admissions </t>
+          <t>MSN Healthcare Solutions (Intellirad)-ADMO</t>
         </is>
       </c>
       <c r="H213" t="inlineStr">
@@ -16730,7 +16730,7 @@
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t xml:space="preserve">MSN Healthcare Solutions (Intellirad)-ITS DI Results </t>
+          <t>MSN Healthcare Solutions (Intellirad)-ITSDIRO</t>
         </is>
       </c>
       <c r="H214" t="inlineStr">
@@ -16874,7 +16874,7 @@
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t xml:space="preserve">McKesson (MPF-Patient Folder/HPF Facility)-ITS HM Results </t>
+          <t>McKesson (MPF-Patient Folder/HPF Facility)-ITSHMRO</t>
         </is>
       </c>
       <c r="H216" t="inlineStr">
@@ -17018,7 +17018,7 @@
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medaxion (Medaxion Pulse to MPF-Patient Folder/HPF Facility)-Scanned Documents </t>
+          <t>Medaxion (Medaxion Pulse to MPF-Patient Folder/HPF Facility)-SCAIMG</t>
         </is>
       </c>
       <c r="H218" t="inlineStr">
@@ -17162,7 +17162,7 @@
       </c>
       <c r="G220" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medaxion (Medaxion Pulse)-Admissions </t>
+          <t>Medaxion (Medaxion Pulse)-ADMO</t>
         </is>
       </c>
       <c r="H220" t="inlineStr">
@@ -17244,7 +17244,7 @@
       </c>
       <c r="G221" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medaxion (Medaxion Pulse)-Scheduling </t>
+          <t>Medaxion (Medaxion Pulse)-CWSO</t>
         </is>
       </c>
       <c r="H221" t="inlineStr">
@@ -17388,7 +17388,7 @@
       </c>
       <c r="G223" t="inlineStr">
         <is>
-          <t>Meditech (HCA 5.6)-</t>
+          <t>Meditech (HCA 5.6)-ADMO</t>
         </is>
       </c>
       <c r="H223" t="inlineStr">
@@ -17434,6 +17434,21 @@
       <c r="P223" t="inlineStr">
         <is>
           <t>Inbound</t>
+        </is>
+      </c>
+      <c r="Q223" t="inlineStr">
+        <is>
+          <t>ADMO</t>
+        </is>
+      </c>
+      <c r="R223" t="inlineStr">
+        <is>
+          <t>ADT</t>
+        </is>
+      </c>
+      <c r="S223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admissions </t>
         </is>
       </c>
     </row>
@@ -17455,7 +17470,7 @@
       </c>
       <c r="G224" t="inlineStr">
         <is>
-          <t xml:space="preserve">Meditech (HCA 5.6)-Admissions </t>
+          <t>Meditech (HCA 5.6)-ITSDIRO</t>
         </is>
       </c>
       <c r="H224" t="inlineStr">
@@ -17505,17 +17520,17 @@
       </c>
       <c r="Q224" t="inlineStr">
         <is>
-          <t>ADMO</t>
+          <t>ITSDIRO</t>
         </is>
       </c>
       <c r="R224" t="inlineStr">
         <is>
-          <t>ADT</t>
+          <t>ORU</t>
         </is>
       </c>
       <c r="S224" t="inlineStr">
         <is>
-          <t xml:space="preserve">Admissions </t>
+          <t xml:space="preserve">ITS DI Results </t>
         </is>
       </c>
     </row>
@@ -17537,7 +17552,7 @@
       </c>
       <c r="G225" t="inlineStr">
         <is>
-          <t xml:space="preserve">Meditech (HCA 5.6)-ITS DI Results </t>
+          <t>Meditech (HCA 5.6)-ITSHMRO</t>
         </is>
       </c>
       <c r="H225" t="inlineStr">
@@ -17587,7 +17602,7 @@
       </c>
       <c r="Q225" t="inlineStr">
         <is>
-          <t>ITSDIRO</t>
+          <t>ITSHMRO</t>
         </is>
       </c>
       <c r="R225" t="inlineStr">
@@ -17597,7 +17612,7 @@
       </c>
       <c r="S225" t="inlineStr">
         <is>
-          <t xml:space="preserve">ITS DI Results </t>
+          <t xml:space="preserve">ITS HM Results </t>
         </is>
       </c>
     </row>
@@ -17619,7 +17634,7 @@
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t xml:space="preserve">Meditech (HCA 5.6)-ITS HM Results </t>
+          <t>Meditech (HCA 5.6)-LABRES</t>
         </is>
       </c>
       <c r="H226" t="inlineStr">
@@ -17669,7 +17684,7 @@
       </c>
       <c r="Q226" t="inlineStr">
         <is>
-          <t>ITSHMRO</t>
+          <t>LABRES</t>
         </is>
       </c>
       <c r="R226" t="inlineStr">
@@ -17679,7 +17694,7 @@
       </c>
       <c r="S226" t="inlineStr">
         <is>
-          <t xml:space="preserve">ITS HM Results </t>
+          <t xml:space="preserve">Lab Results (Discrete) </t>
         </is>
       </c>
     </row>
@@ -17701,7 +17716,7 @@
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t xml:space="preserve">Meditech (HCA 5.6)-Lab Results (Discrete) </t>
+          <t>Meditech (HCA 5.6)-LABRES2</t>
         </is>
       </c>
       <c r="H227" t="inlineStr">
@@ -17751,7 +17766,7 @@
       </c>
       <c r="Q227" t="inlineStr">
         <is>
-          <t>LABRES</t>
+          <t>LABRES2</t>
         </is>
       </c>
       <c r="R227" t="inlineStr">
@@ -17761,7 +17776,7 @@
       </c>
       <c r="S227" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lab Results (Discrete) </t>
+          <t>Pathology Results</t>
         </is>
       </c>
     </row>
@@ -17783,7 +17798,7 @@
       </c>
       <c r="G228" t="inlineStr">
         <is>
-          <t xml:space="preserve">Meditech (HCA 5.6)-OM Orders </t>
+          <t>Meditech (HCA 5.6)-OMORDO</t>
         </is>
       </c>
       <c r="H228" t="inlineStr">
@@ -17865,7 +17880,7 @@
       </c>
       <c r="G229" t="inlineStr">
         <is>
-          <t>Meditech (HCA 5.6)-Pathology Results</t>
+          <t>Meditech (HCA 5.6)-PHAORD</t>
         </is>
       </c>
       <c r="H229" t="inlineStr">
@@ -17915,17 +17930,17 @@
       </c>
       <c r="Q229" t="inlineStr">
         <is>
-          <t>LABRES2</t>
+          <t>PHAORD</t>
         </is>
       </c>
       <c r="R229" t="inlineStr">
         <is>
-          <t>ORU</t>
+          <t>RDE</t>
         </is>
       </c>
       <c r="S229" t="inlineStr">
         <is>
-          <t>Pathology Results</t>
+          <t xml:space="preserve">Pharmacy Orders </t>
         </is>
       </c>
     </row>
@@ -17947,7 +17962,7 @@
       </c>
       <c r="G230" t="inlineStr">
         <is>
-          <t xml:space="preserve">Meditech (HCA 5.6)-Pharmacy Orders </t>
+          <t>Meditech (HCA 5.6)-radord</t>
         </is>
       </c>
       <c r="H230" t="inlineStr">
@@ -17993,21 +18008,6 @@
       <c r="P230" t="inlineStr">
         <is>
           <t>Inbound</t>
-        </is>
-      </c>
-      <c r="Q230" t="inlineStr">
-        <is>
-          <t>PHAORD</t>
-        </is>
-      </c>
-      <c r="R230" t="inlineStr">
-        <is>
-          <t>RDE</t>
-        </is>
-      </c>
-      <c r="S230" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pharmacy Orders </t>
         </is>
       </c>
     </row>
@@ -18091,7 +18091,7 @@
       </c>
       <c r="G232" t="inlineStr">
         <is>
-          <t xml:space="preserve">Meditech (MPF-Patient Folder/HPF Facility)-Admissions </t>
+          <t>Meditech (MPF-Patient Folder/HPF Facility)-ADMO</t>
         </is>
       </c>
       <c r="H232" t="inlineStr">
@@ -18173,7 +18173,7 @@
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Meditech (MPF-Patient Folder/HPF Facility)-ITS DI Results </t>
+          <t>Meditech (MPF-Patient Folder/HPF Facility)-ITSDIRO</t>
         </is>
       </c>
       <c r="H233" t="inlineStr">
@@ -18255,7 +18255,7 @@
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t xml:space="preserve">Meditech (MPF-Patient Folder/HPF Facility)-ITS HM Results </t>
+          <t>Meditech (MPF-Patient Folder/HPF Facility)-ITSHMRO</t>
         </is>
       </c>
       <c r="H234" t="inlineStr">
@@ -18337,7 +18337,7 @@
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t xml:space="preserve">Meditech (MPF-Patient Folder/HPF Facility)-Scanned Documents </t>
+          <t>Meditech (MPF-Patient Folder/HPF Facility)-SCAIMG</t>
         </is>
       </c>
       <c r="H235" t="inlineStr">
@@ -18481,7 +18481,7 @@
       </c>
       <c r="G237" t="inlineStr">
         <is>
-          <t xml:space="preserve">Midas+ (Care Management-Facility)-Admissions </t>
+          <t>Midas+ (Care Management-Facility)-ADMO</t>
         </is>
       </c>
       <c r="H237" t="inlineStr">
@@ -18563,7 +18563,7 @@
       </c>
       <c r="G238" t="inlineStr">
         <is>
-          <t xml:space="preserve">Midas+ (Care Management-Facility)-Admissions </t>
+          <t>Midas+ (Care Management-Facility)-ADMO</t>
         </is>
       </c>
       <c r="H238" t="inlineStr">
@@ -18645,7 +18645,7 @@
       </c>
       <c r="G239" t="inlineStr">
         <is>
-          <t xml:space="preserve">Midas+ (Care Management-Facility)-ITS DI Results </t>
+          <t>Midas+ (Care Management-Facility)-ITSDIRO</t>
         </is>
       </c>
       <c r="H239" t="inlineStr">
@@ -18727,7 +18727,7 @@
       </c>
       <c r="G240" t="inlineStr">
         <is>
-          <t xml:space="preserve">Midas+ (Care Management-Facility)-ITS HM Results </t>
+          <t>Midas+ (Care Management-Facility)-ITSHMRO</t>
         </is>
       </c>
       <c r="H240" t="inlineStr">
@@ -18809,7 +18809,7 @@
       </c>
       <c r="G241" t="inlineStr">
         <is>
-          <t xml:space="preserve">Midas+ (Care Management-Facility)-ITS HM Results </t>
+          <t>Midas+ (Care Management-Facility)-ITSHMRO</t>
         </is>
       </c>
       <c r="H241" t="inlineStr">
@@ -18953,7 +18953,7 @@
       </c>
       <c r="G243" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mobile Heartbeat (imobile)-Admissions </t>
+          <t>Mobile Heartbeat (imobile)-ADMO</t>
         </is>
       </c>
       <c r="H243" t="inlineStr">
@@ -19035,7 +19035,7 @@
       </c>
       <c r="G244" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mobile Heartbeat (imobile)-Lab Results (Discrete) </t>
+          <t>Mobile Heartbeat (imobile)-LABRES</t>
         </is>
       </c>
       <c r="H244" t="inlineStr">
@@ -19179,7 +19179,7 @@
       </c>
       <c r="G246" t="inlineStr">
         <is>
-          <t xml:space="preserve">Net Health (ReDoc Xfit)-Admissions </t>
+          <t>Net Health (ReDoc Xfit)-ADMO</t>
         </is>
       </c>
       <c r="H246" t="inlineStr">
@@ -19261,7 +19261,7 @@
       </c>
       <c r="G247" t="inlineStr">
         <is>
-          <t xml:space="preserve">Net Health (ReDoc Xfit)-Charges </t>
+          <t>Net Health (ReDoc Xfit)-ITSHMRO</t>
         </is>
       </c>
       <c r="H247" t="inlineStr">
@@ -19311,17 +19311,17 @@
       </c>
       <c r="Q247" t="inlineStr">
         <is>
-          <t>Patient Accounting</t>
+          <t>ITSHMRO</t>
         </is>
       </c>
       <c r="R247" t="inlineStr">
         <is>
-          <t>DFT</t>
+          <t>ORU</t>
         </is>
       </c>
       <c r="S247" t="inlineStr">
         <is>
-          <t xml:space="preserve">Charges </t>
+          <t xml:space="preserve">ITS HM Results </t>
         </is>
       </c>
     </row>
@@ -19343,7 +19343,7 @@
       </c>
       <c r="G248" t="inlineStr">
         <is>
-          <t xml:space="preserve">Net Health (ReDoc Xfit)-ITS HM Results </t>
+          <t>Net Health (ReDoc Xfit)-OMORDO</t>
         </is>
       </c>
       <c r="H248" t="inlineStr">
@@ -19388,22 +19388,22 @@
       </c>
       <c r="P248" t="inlineStr">
         <is>
-          <t>Inbound</t>
+          <t>Outbound</t>
         </is>
       </c>
       <c r="Q248" t="inlineStr">
         <is>
-          <t>ITSHMRO</t>
+          <t>OMORDO</t>
         </is>
       </c>
       <c r="R248" t="inlineStr">
         <is>
-          <t>ORU</t>
+          <t>ORM</t>
         </is>
       </c>
       <c r="S248" t="inlineStr">
         <is>
-          <t xml:space="preserve">ITS HM Results </t>
+          <t xml:space="preserve">OM Orders </t>
         </is>
       </c>
     </row>
@@ -19425,7 +19425,7 @@
       </c>
       <c r="G249" t="inlineStr">
         <is>
-          <t xml:space="preserve">Net Health (ReDoc Xfit)-OM Orders </t>
+          <t>Net Health (ReDoc Xfit)-Patient Accounting</t>
         </is>
       </c>
       <c r="H249" t="inlineStr">
@@ -19470,22 +19470,22 @@
       </c>
       <c r="P249" t="inlineStr">
         <is>
-          <t>Outbound</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="Q249" t="inlineStr">
         <is>
-          <t>OMORDO</t>
+          <t>Patient Accounting</t>
         </is>
       </c>
       <c r="R249" t="inlineStr">
         <is>
-          <t>ORM</t>
+          <t>DFT</t>
         </is>
       </c>
       <c r="S249" t="inlineStr">
         <is>
-          <t xml:space="preserve">OM Orders </t>
+          <t xml:space="preserve">Charges </t>
         </is>
       </c>
     </row>
@@ -19569,7 +19569,7 @@
       </c>
       <c r="G251" t="inlineStr">
         <is>
-          <t xml:space="preserve">Net Health (Wound Care)-Admissions </t>
+          <t>Net Health (Wound Care)-ADMO</t>
         </is>
       </c>
       <c r="H251" t="inlineStr">
@@ -19713,7 +19713,7 @@
       </c>
       <c r="G253" t="inlineStr">
         <is>
-          <t xml:space="preserve">Netsmart (UDS PROi to MPF-Patient Folder/HPF Facility)-ITS HM Results </t>
+          <t>Netsmart (UDS PROi to MPF-Patient Folder/HPF Facility)-ITSHMRO</t>
         </is>
       </c>
       <c r="H253" t="inlineStr">
@@ -19857,7 +19857,7 @@
       </c>
       <c r="G255" t="inlineStr">
         <is>
-          <t>Netsmart (UDS PROi to PA)-Case Mix Group</t>
+          <t>Netsmart (UDS PROi to PA)-nan</t>
         </is>
       </c>
       <c r="H255" t="inlineStr">
@@ -19996,7 +19996,7 @@
       </c>
       <c r="G257" t="inlineStr">
         <is>
-          <t xml:space="preserve">Netsmart (UDS PROi)-Admissions </t>
+          <t>Netsmart (UDS PROi)-ADMO</t>
         </is>
       </c>
       <c r="H257" t="inlineStr">
@@ -20078,7 +20078,7 @@
       </c>
       <c r="G258" t="inlineStr">
         <is>
-          <t xml:space="preserve">Netsmart (UDS PROi)-Admissions </t>
+          <t>Netsmart (UDS PROi)-ADMO</t>
         </is>
       </c>
       <c r="H258" t="inlineStr">
@@ -20222,7 +20222,7 @@
       </c>
       <c r="G260" t="inlineStr">
         <is>
-          <t>Nuance (Primordial)-</t>
+          <t>Nuance (Primordial)-ADMO</t>
         </is>
       </c>
       <c r="H260" t="inlineStr">
@@ -20268,6 +20268,21 @@
       <c r="P260" t="inlineStr">
         <is>
           <t>Outbound</t>
+        </is>
+      </c>
+      <c r="Q260" t="inlineStr">
+        <is>
+          <t>ADMO</t>
+        </is>
+      </c>
+      <c r="R260" t="inlineStr">
+        <is>
+          <t>ADT</t>
+        </is>
+      </c>
+      <c r="S260" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admissions </t>
         </is>
       </c>
     </row>
@@ -20289,7 +20304,7 @@
       </c>
       <c r="G261" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nuance (Primordial)-Admissions </t>
+          <t>Nuance (Primordial)-ITSDIRO</t>
         </is>
       </c>
       <c r="H261" t="inlineStr">
@@ -20339,17 +20354,17 @@
       </c>
       <c r="Q261" t="inlineStr">
         <is>
-          <t>ADMO</t>
+          <t>ITSDIRO</t>
         </is>
       </c>
       <c r="R261" t="inlineStr">
         <is>
-          <t>ADT</t>
+          <t>ORU</t>
         </is>
       </c>
       <c r="S261" t="inlineStr">
         <is>
-          <t xml:space="preserve">Admissions </t>
+          <t xml:space="preserve">ITS DI Results </t>
         </is>
       </c>
     </row>
@@ -20371,7 +20386,7 @@
       </c>
       <c r="G262" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nuance (Primordial)-ITS DI Results </t>
+          <t>Nuance (Primordial)-radord</t>
         </is>
       </c>
       <c r="H262" t="inlineStr">
@@ -20417,21 +20432,6 @@
       <c r="P262" t="inlineStr">
         <is>
           <t>Outbound</t>
-        </is>
-      </c>
-      <c r="Q262" t="inlineStr">
-        <is>
-          <t>ITSDIRO</t>
-        </is>
-      </c>
-      <c r="R262" t="inlineStr">
-        <is>
-          <t>ORU</t>
-        </is>
-      </c>
-      <c r="S262" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ITS DI Results </t>
         </is>
       </c>
     </row>
@@ -20515,7 +20515,7 @@
       </c>
       <c r="G264" t="inlineStr">
         <is>
-          <t>Omnicell (Optiflex to SMART)-</t>
+          <t>Omnicell (Optiflex to SMART)-mmrepl</t>
         </is>
       </c>
       <c r="H264" t="inlineStr">
@@ -20644,7 +20644,7 @@
       </c>
       <c r="G266" t="inlineStr">
         <is>
-          <t xml:space="preserve">Omnicell (Optiflex)-Admissions </t>
+          <t>Omnicell (Optiflex)-ADMO</t>
         </is>
       </c>
       <c r="H266" t="inlineStr">
@@ -20726,7 +20726,7 @@
       </c>
       <c r="G267" t="inlineStr">
         <is>
-          <t xml:space="preserve">Omnicell (Optiflex)-Charges </t>
+          <t>Omnicell (Optiflex)-Patient Accounting</t>
         </is>
       </c>
       <c r="H267" t="inlineStr">
@@ -20870,7 +20870,7 @@
       </c>
       <c r="G269" t="inlineStr">
         <is>
-          <t xml:space="preserve">Passport Health Communications, Inc. (eCare Next)-Admissions </t>
+          <t>Passport Health Communications, Inc. (eCare Next)-ADMO</t>
         </is>
       </c>
       <c r="H269" t="inlineStr">
@@ -21014,7 +21014,7 @@
       </c>
       <c r="G271" t="inlineStr">
         <is>
-          <t>Patient Keeper (Portal)-</t>
+          <t>Patient Keeper (Portal)-ITSHMRO</t>
         </is>
       </c>
       <c r="H271" t="inlineStr">
@@ -21060,6 +21060,21 @@
       <c r="P271" t="inlineStr">
         <is>
           <t>Inbound</t>
+        </is>
+      </c>
+      <c r="Q271" t="inlineStr">
+        <is>
+          <t>ITSHMRO</t>
+        </is>
+      </c>
+      <c r="R271" t="inlineStr">
+        <is>
+          <t>ORU</t>
+        </is>
+      </c>
+      <c r="S271" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ITS HM Results </t>
         </is>
       </c>
     </row>
@@ -21081,7 +21096,7 @@
       </c>
       <c r="G272" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patient Keeper (Portal)-ITS HM Results </t>
+          <t>Patient Keeper (Portal)-eps</t>
         </is>
       </c>
       <c r="H272" t="inlineStr">
@@ -21127,21 +21142,6 @@
       <c r="P272" t="inlineStr">
         <is>
           <t>Inbound</t>
-        </is>
-      </c>
-      <c r="Q272" t="inlineStr">
-        <is>
-          <t>ITSHMRO</t>
-        </is>
-      </c>
-      <c r="R272" t="inlineStr">
-        <is>
-          <t>ORU</t>
-        </is>
-      </c>
-      <c r="S272" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ITS HM Results </t>
         </is>
       </c>
     </row>
@@ -21225,7 +21225,7 @@
       </c>
       <c r="G274" t="inlineStr">
         <is>
-          <t>Provation (Apex to MPF-Patient Folder/HPF Facility)-</t>
+          <t>Provation (Apex to MPF-Patient Folder/HPF Facility)-imgurl</t>
         </is>
       </c>
       <c r="H274" t="inlineStr">
@@ -21354,7 +21354,7 @@
       </c>
       <c r="G276" t="inlineStr">
         <is>
-          <t xml:space="preserve">Provation (Apex)-Admissions </t>
+          <t>Provation (Apex)-ADMO</t>
         </is>
       </c>
       <c r="H276" t="inlineStr">
@@ -21436,7 +21436,7 @@
       </c>
       <c r="G277" t="inlineStr">
         <is>
-          <t xml:space="preserve">Provation (Apex)-ITS HM Results </t>
+          <t>Provation (Apex)-CWSO</t>
         </is>
       </c>
       <c r="H277" t="inlineStr">
@@ -21481,22 +21481,22 @@
       </c>
       <c r="P277" t="inlineStr">
         <is>
-          <t>Inbound</t>
+          <t>Outbound</t>
         </is>
       </c>
       <c r="Q277" t="inlineStr">
         <is>
-          <t>ITSHMRO</t>
+          <t>CWSO</t>
         </is>
       </c>
       <c r="R277" t="inlineStr">
         <is>
-          <t>ORU</t>
+          <t>SIU</t>
         </is>
       </c>
       <c r="S277" t="inlineStr">
         <is>
-          <t xml:space="preserve">ITS HM Results </t>
+          <t xml:space="preserve">Scheduling </t>
         </is>
       </c>
     </row>
@@ -21518,7 +21518,7 @@
       </c>
       <c r="G278" t="inlineStr">
         <is>
-          <t xml:space="preserve">Provation (Apex)-Scheduling </t>
+          <t>Provation (Apex)-ITSHMRO</t>
         </is>
       </c>
       <c r="H278" t="inlineStr">
@@ -21563,22 +21563,22 @@
       </c>
       <c r="P278" t="inlineStr">
         <is>
-          <t>Outbound</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="Q278" t="inlineStr">
         <is>
-          <t>CWSO</t>
+          <t>ITSHMRO</t>
         </is>
       </c>
       <c r="R278" t="inlineStr">
         <is>
-          <t>SIU</t>
+          <t>ORU</t>
         </is>
       </c>
       <c r="S278" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scheduling </t>
+          <t xml:space="preserve">ITS HM Results </t>
         </is>
       </c>
     </row>
@@ -21662,7 +21662,7 @@
       </c>
       <c r="G280" t="inlineStr">
         <is>
-          <t xml:space="preserve">Provation (MD - CMORE to MD - CMORE)-ITS HM Results </t>
+          <t>Provation (MD - CMORE to MD - CMORE)-ITSHMRO</t>
         </is>
       </c>
       <c r="H280" t="inlineStr">
@@ -21806,7 +21806,7 @@
       </c>
       <c r="G282" t="inlineStr">
         <is>
-          <t xml:space="preserve">Provation (MD - CMORE to MPF-Patient Folder/HPF Facility)-Scanned Documents </t>
+          <t>Provation (MD - CMORE to MPF-Patient Folder/HPF Facility)-SCAIMG</t>
         </is>
       </c>
       <c r="H282" t="inlineStr">
@@ -21950,7 +21950,7 @@
       </c>
       <c r="G284" t="inlineStr">
         <is>
-          <t xml:space="preserve">Provation (MD - CMORE)-Admissions </t>
+          <t>Provation (MD - CMORE)-ADMO</t>
         </is>
       </c>
       <c r="H284" t="inlineStr">
@@ -22032,7 +22032,7 @@
       </c>
       <c r="G285" t="inlineStr">
         <is>
-          <t xml:space="preserve">Provation (MD - CMORE)-ITS HM Results </t>
+          <t>Provation (MD - CMORE)-ITSHMRO</t>
         </is>
       </c>
       <c r="H285" t="inlineStr">
@@ -22176,7 +22176,7 @@
       </c>
       <c r="G287" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rauland (Responder)-Admissions </t>
+          <t>Rauland (Responder)-ADMO</t>
         </is>
       </c>
       <c r="H287" t="inlineStr">
@@ -22320,7 +22320,7 @@
       </c>
       <c r="G289" t="inlineStr">
         <is>
-          <t>Telcor (Quick-Link)-</t>
+          <t>Telcor (Quick-Link)-ADMO</t>
         </is>
       </c>
       <c r="H289" t="inlineStr">
@@ -22365,7 +22365,22 @@
       </c>
       <c r="P289" t="inlineStr">
         <is>
-          <t>Inbound</t>
+          <t>Outbound</t>
+        </is>
+      </c>
+      <c r="Q289" t="inlineStr">
+        <is>
+          <t>ADMO</t>
+        </is>
+      </c>
+      <c r="R289" t="inlineStr">
+        <is>
+          <t>ADT</t>
+        </is>
+      </c>
+      <c r="S289" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admissions </t>
         </is>
       </c>
     </row>
@@ -22387,7 +22402,7 @@
       </c>
       <c r="G290" t="inlineStr">
         <is>
-          <t xml:space="preserve">Telcor (Quick-Link)-Admissions </t>
+          <t>Telcor (Quick-Link)-labpoc</t>
         </is>
       </c>
       <c r="H290" t="inlineStr">
@@ -22432,22 +22447,7 @@
       </c>
       <c r="P290" t="inlineStr">
         <is>
-          <t>Outbound</t>
-        </is>
-      </c>
-      <c r="Q290" t="inlineStr">
-        <is>
-          <t>ADMO</t>
-        </is>
-      </c>
-      <c r="R290" t="inlineStr">
-        <is>
-          <t>ADT</t>
-        </is>
-      </c>
-      <c r="S290" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Admissions </t>
+          <t>Inbound</t>
         </is>
       </c>
     </row>
@@ -22531,7 +22531,7 @@
       </c>
       <c r="G292" t="inlineStr">
         <is>
-          <t xml:space="preserve">TeleSpecialists (TeleCare)-Admissions </t>
+          <t>TeleSpecialists (TeleCare)-ADMO</t>
         </is>
       </c>
       <c r="H292" t="inlineStr">
@@ -22613,7 +22613,7 @@
       </c>
       <c r="G293" t="inlineStr">
         <is>
-          <t xml:space="preserve">TeleSpecialists (TeleCare)-ITS HM Results </t>
+          <t>TeleSpecialists (TeleCare)-ITSHMRO</t>
         </is>
       </c>
       <c r="H293" t="inlineStr">
@@ -22695,7 +22695,7 @@
       </c>
       <c r="G294" t="inlineStr">
         <is>
-          <t xml:space="preserve">TeleSpecialists (TeleCare)-OM Orders </t>
+          <t>TeleSpecialists (TeleCare)-OMORDO</t>
         </is>
       </c>
       <c r="H294" t="inlineStr">
@@ -22839,7 +22839,7 @@
       </c>
       <c r="G296" t="inlineStr">
         <is>
-          <t xml:space="preserve">TeleTracking (TransferCenter IQ)-Admissions </t>
+          <t>TeleTracking (TransferCenter IQ)-ADMO</t>
         </is>
       </c>
       <c r="H296" t="inlineStr">
@@ -22921,7 +22921,7 @@
       </c>
       <c r="G297" t="inlineStr">
         <is>
-          <t xml:space="preserve">TeleTracking (TransferCenter IQ)-OM Orders </t>
+          <t>TeleTracking (TransferCenter IQ)-OMORDO</t>
         </is>
       </c>
       <c r="H297" t="inlineStr">
@@ -23003,7 +23003,7 @@
       </c>
       <c r="G298" t="inlineStr">
         <is>
-          <t>TeleTracking (TransferCenter IQ)-iPeople Nursing Assessment Forms</t>
+          <t>TeleTracking (TransferCenter IQ)-iPeople PCS</t>
         </is>
       </c>
       <c r="H298" t="inlineStr">
@@ -23147,7 +23147,7 @@
       </c>
       <c r="G300" t="inlineStr">
         <is>
-          <t xml:space="preserve">Telexy Healthcare Inc (Q-path)-Admissions </t>
+          <t>Telexy Healthcare Inc (Q-path)-ADMO</t>
         </is>
       </c>
       <c r="H300" t="inlineStr">
@@ -23291,7 +23291,7 @@
       </c>
       <c r="G302" t="inlineStr">
         <is>
-          <t>Ventana Medical Systems (VANTAGE)-</t>
+          <t>Ventana Medical Systems (VANTAGE)-pthord</t>
         </is>
       </c>
       <c r="H302" t="inlineStr">
@@ -23420,7 +23420,7 @@
       </c>
       <c r="G304" t="inlineStr">
         <is>
-          <t xml:space="preserve">VigiLanz Corp (Dynamic PharmacoVigilance-Facility)-Admissions </t>
+          <t>VigiLanz Corp (Dynamic PharmacoVigilance-Facility)-ADMO</t>
         </is>
       </c>
       <c r="H304" t="inlineStr">
@@ -23502,7 +23502,7 @@
       </c>
       <c r="G305" t="inlineStr">
         <is>
-          <t xml:space="preserve">VigiLanz Corp (Dynamic PharmacoVigilance-Facility)-ITS DI Results </t>
+          <t>VigiLanz Corp (Dynamic PharmacoVigilance-Facility)-ITSDIRO</t>
         </is>
       </c>
       <c r="H305" t="inlineStr">
@@ -23584,7 +23584,7 @@
       </c>
       <c r="G306" t="inlineStr">
         <is>
-          <t xml:space="preserve">VigiLanz Corp (Dynamic PharmacoVigilance-Facility)-Lab Results (Discrete) </t>
+          <t>VigiLanz Corp (Dynamic PharmacoVigilance-Facility)-LABRES</t>
         </is>
       </c>
       <c r="H306" t="inlineStr">
@@ -23666,7 +23666,7 @@
       </c>
       <c r="G307" t="inlineStr">
         <is>
-          <t xml:space="preserve">VigiLanz Corp (Dynamic PharmacoVigilance-Facility)-OM Orders </t>
+          <t>VigiLanz Corp (Dynamic PharmacoVigilance-Facility)-OMORDO</t>
         </is>
       </c>
       <c r="H307" t="inlineStr">
@@ -23748,7 +23748,7 @@
       </c>
       <c r="G308" t="inlineStr">
         <is>
-          <t xml:space="preserve">VigiLanz Corp (Dynamic PharmacoVigilance-Facility)-OM Orders </t>
+          <t>VigiLanz Corp (Dynamic PharmacoVigilance-Facility)-OMORDO</t>
         </is>
       </c>
       <c r="H308" t="inlineStr">
@@ -23830,7 +23830,7 @@
       </c>
       <c r="G309" t="inlineStr">
         <is>
-          <t xml:space="preserve">VigiLanz Corp (Dynamic PharmacoVigilance-Facility)-Pharmacy Orders </t>
+          <t>VigiLanz Corp (Dynamic PharmacoVigilance-Facility)-PHAORD</t>
         </is>
       </c>
       <c r="H309" t="inlineStr">
@@ -23974,7 +23974,7 @@
       </c>
       <c r="G311" t="inlineStr">
         <is>
-          <t>Volpara Health (Aspen Breast)-</t>
+          <t>Volpara Health (Aspen Breast)-radord</t>
         </is>
       </c>
       <c r="H311" t="inlineStr">
@@ -24103,7 +24103,7 @@
       </c>
       <c r="G313" t="inlineStr">
         <is>
-          <t>dbMotion (db Motion)-</t>
+          <t>dbMotion (db Motion)-ADMO</t>
         </is>
       </c>
       <c r="H313" t="inlineStr">
@@ -24149,6 +24149,21 @@
       <c r="P313" t="inlineStr">
         <is>
           <t>Outbound</t>
+        </is>
+      </c>
+      <c r="Q313" t="inlineStr">
+        <is>
+          <t>ADMO</t>
+        </is>
+      </c>
+      <c r="R313" t="inlineStr">
+        <is>
+          <t>ADT</t>
+        </is>
+      </c>
+      <c r="S313" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admissions </t>
         </is>
       </c>
     </row>
@@ -24170,7 +24185,7 @@
       </c>
       <c r="G314" t="inlineStr">
         <is>
-          <t xml:space="preserve">dbMotion (db Motion)-Admissions </t>
+          <t>dbMotion (db Motion)-IMMUN</t>
         </is>
       </c>
       <c r="H314" t="inlineStr">
@@ -24220,17 +24235,17 @@
       </c>
       <c r="Q314" t="inlineStr">
         <is>
-          <t>ADMO</t>
+          <t>IMMUN</t>
         </is>
       </c>
       <c r="R314" t="inlineStr">
         <is>
-          <t>ADT</t>
+          <t>VXU</t>
         </is>
       </c>
       <c r="S314" t="inlineStr">
         <is>
-          <t xml:space="preserve">Admissions </t>
+          <t>MU-Immunizations</t>
         </is>
       </c>
     </row>
@@ -24252,7 +24267,7 @@
       </c>
       <c r="G315" t="inlineStr">
         <is>
-          <t xml:space="preserve">dbMotion (db Motion)-ITS DI Results </t>
+          <t>dbMotion (db Motion)-ITSDIRO</t>
         </is>
       </c>
       <c r="H315" t="inlineStr">
@@ -24334,7 +24349,7 @@
       </c>
       <c r="G316" t="inlineStr">
         <is>
-          <t xml:space="preserve">dbMotion (db Motion)-ITS HM Results </t>
+          <t>dbMotion (db Motion)-ITSHMRO</t>
         </is>
       </c>
       <c r="H316" t="inlineStr">
@@ -24416,7 +24431,7 @@
       </c>
       <c r="G317" t="inlineStr">
         <is>
-          <t xml:space="preserve">dbMotion (db Motion)-Lab Results (Discrete) </t>
+          <t>dbMotion (db Motion)-LABRES</t>
         </is>
       </c>
       <c r="H317" t="inlineStr">
@@ -24498,7 +24513,7 @@
       </c>
       <c r="G318" t="inlineStr">
         <is>
-          <t>dbMotion (db Motion)-MU-Immunizations</t>
+          <t>dbMotion (db Motion)-LABRES2</t>
         </is>
       </c>
       <c r="H318" t="inlineStr">
@@ -24548,17 +24563,17 @@
       </c>
       <c r="Q318" t="inlineStr">
         <is>
-          <t>IMMUN</t>
+          <t>LABRES2</t>
         </is>
       </c>
       <c r="R318" t="inlineStr">
         <is>
-          <t>VXU</t>
+          <t>ORU</t>
         </is>
       </c>
       <c r="S318" t="inlineStr">
         <is>
-          <t>MU-Immunizations</t>
+          <t>Pathology Results</t>
         </is>
       </c>
     </row>
@@ -24580,7 +24595,7 @@
       </c>
       <c r="G319" t="inlineStr">
         <is>
-          <t>dbMotion (db Motion)-Pathology Results</t>
+          <t>dbMotion (db Motion)-PHAORD</t>
         </is>
       </c>
       <c r="H319" t="inlineStr">
@@ -24630,17 +24645,17 @@
       </c>
       <c r="Q319" t="inlineStr">
         <is>
-          <t>LABRES2</t>
+          <t>PHAORD</t>
         </is>
       </c>
       <c r="R319" t="inlineStr">
         <is>
-          <t>ORU</t>
+          <t>RDE</t>
         </is>
       </c>
       <c r="S319" t="inlineStr">
         <is>
-          <t>Pathology Results</t>
+          <t xml:space="preserve">Pharmacy Orders </t>
         </is>
       </c>
     </row>
@@ -24662,7 +24677,7 @@
       </c>
       <c r="G320" t="inlineStr">
         <is>
-          <t xml:space="preserve">dbMotion (db Motion)-Pharmacy Orders </t>
+          <t>dbMotion (db Motion)-iPeople EDM</t>
         </is>
       </c>
       <c r="H320" t="inlineStr">
@@ -24712,17 +24727,17 @@
       </c>
       <c r="Q320" t="inlineStr">
         <is>
-          <t>PHAORD</t>
+          <t>iPeople EDM</t>
         </is>
       </c>
       <c r="R320" t="inlineStr">
         <is>
-          <t>RDE</t>
+          <t>EDM - iPeople</t>
         </is>
       </c>
       <c r="S320" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pharmacy Orders </t>
+          <t>iPeople ED Patient Visit Data</t>
         </is>
       </c>
     </row>
@@ -24744,7 +24759,7 @@
       </c>
       <c r="G321" t="inlineStr">
         <is>
-          <t>dbMotion (db Motion)-iPeople ED Patient Visit Data</t>
+          <t>dbMotion (db Motion)-iPeople PCS</t>
         </is>
       </c>
       <c r="H321" t="inlineStr">
@@ -24794,17 +24809,17 @@
       </c>
       <c r="Q321" t="inlineStr">
         <is>
-          <t>iPeople EDM</t>
+          <t>iPeople PCS</t>
         </is>
       </c>
       <c r="R321" t="inlineStr">
         <is>
-          <t>EDM - iPeople</t>
+          <t>PCS - iPeople</t>
         </is>
       </c>
       <c r="S321" t="inlineStr">
         <is>
-          <t>iPeople ED Patient Visit Data</t>
+          <t>iPeople Nursing Assessment Forms</t>
         </is>
       </c>
     </row>
@@ -24826,7 +24841,7 @@
       </c>
       <c r="G322" t="inlineStr">
         <is>
-          <t>dbMotion (db Motion)-iPeople Nursing Assessment Forms</t>
+          <t>dbMotion (db Motion)-radord</t>
         </is>
       </c>
       <c r="H322" t="inlineStr">
@@ -24872,21 +24887,6 @@
       <c r="P322" t="inlineStr">
         <is>
           <t>Outbound</t>
-        </is>
-      </c>
-      <c r="Q322" t="inlineStr">
-        <is>
-          <t>iPeople PCS</t>
-        </is>
-      </c>
-      <c r="R322" t="inlineStr">
-        <is>
-          <t>PCS - iPeople</t>
-        </is>
-      </c>
-      <c r="S322" t="inlineStr">
-        <is>
-          <t>iPeople Nursing Assessment Forms</t>
         </is>
       </c>
     </row>
@@ -24970,7 +24970,7 @@
       </c>
       <c r="G324" t="inlineStr">
         <is>
-          <t>iPeople (HCA 5.6)-iPeople ED Patient Visit Data</t>
+          <t>iPeople (HCA 5.6)-iPeople EDM</t>
         </is>
       </c>
       <c r="H324" t="inlineStr">
@@ -25052,7 +25052,7 @@
       </c>
       <c r="G325" t="inlineStr">
         <is>
-          <t>iPeople (HCA 5.6)-iPeople Medication Administration</t>
+          <t>iPeople (HCA 5.6)-iPeople Meds</t>
         </is>
       </c>
       <c r="H325" t="inlineStr">
@@ -25196,7 +25196,7 @@
       </c>
       <c r="G327" t="inlineStr">
         <is>
-          <t xml:space="preserve">iPeople (iPeople MT56)-OM Orders </t>
+          <t>iPeople (iPeople MT56)-OMORDO</t>
         </is>
       </c>
       <c r="H327" t="inlineStr">
@@ -25278,7 +25278,7 @@
       </c>
       <c r="G328" t="inlineStr">
         <is>
-          <t>iPeople (iPeople MT56)-iPeople ED Patient Visit Data</t>
+          <t>iPeople (iPeople MT56)-iPeople EDM</t>
         </is>
       </c>
       <c r="H328" t="inlineStr">
@@ -25360,7 +25360,7 @@
       </c>
       <c r="G329" t="inlineStr">
         <is>
-          <t>iPeople (iPeople MT56)-iPeople Medication Administration</t>
+          <t>iPeople (iPeople MT56)-iPeople Meds</t>
         </is>
       </c>
       <c r="H329" t="inlineStr">
@@ -25442,7 +25442,7 @@
       </c>
       <c r="G330" t="inlineStr">
         <is>
-          <t>iPeople (iPeople MT56)-iPeople Nursing Assessment Forms</t>
+          <t>iPeople (iPeople MT56)-iPeople PCS</t>
         </is>
       </c>
       <c r="H330" t="inlineStr">

</xml_diff>